<commit_message>
WeeklyPay rotation engine update + workspace cleanup (Nov 6, 2025)
</commit_message>
<xml_diff>
--- a/Etrade_Rollover_IRA_data.xlsx
+++ b/Etrade_Rollover_IRA_data.xlsx
@@ -454,7 +454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA34"/>
+  <dimension ref="A1:AA40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -629,25 +629,25 @@
         </is>
       </c>
       <c r="J2" t="n">
-        <v>63</v>
+        <v>-89.25</v>
       </c>
       <c r="K2" t="n">
-        <v>0.5102</v>
+        <v>-0.7179</v>
       </c>
       <c r="L2" t="n">
-        <v>12411</v>
+        <v>12342.75</v>
       </c>
       <c r="M2" t="n">
         <v>14441.5992</v>
       </c>
       <c r="N2" t="n">
-        <v>-2030.5992</v>
+        <v>-2098.8492</v>
       </c>
       <c r="O2" t="n">
-        <v>-14.0607</v>
+        <v>-14.5333</v>
       </c>
       <c r="P2" t="n">
-        <v>4.5137</v>
+        <v>4.2793</v>
       </c>
       <c r="Q2" t="n">
         <v>13.7539</v>
@@ -665,7 +665,7 @@
         <v>0</v>
       </c>
       <c r="V2" t="n">
-        <v>11.76</v>
+        <v>11.84</v>
       </c>
       <c r="W2" t="inlineStr">
         <is>
@@ -684,25 +684,25 @@
       </c>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>{'lastTrade': 11.82, 'lastTradeTime': 1754683800, 'change': 0.06, 'changePct': 0.5102, 'volume': 1526466, 'quoteStatus': 'CLOSING'}</t>
+          <t>{'lastTrade': 11.755, 'lastTradeTime': 1757527582, 'change': -0.085, 'changePct': -0.7179, 'volume': 711891, 'quoteStatus': 'REALTIME'}</t>
         </is>
       </c>
       <c r="AA2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>429040063900</v>
+        <v>413847387900</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>PSTG</t>
+          <t>QDTE</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1738731600000</v>
+        <v>1732165200000</v>
       </c>
       <c r="D3" t="n">
-        <v>69.1527</v>
+        <v>38.4982</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
@@ -711,7 +711,7 @@
         <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>200</v>
+        <v>304</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -724,28 +724,28 @@
         </is>
       </c>
       <c r="J3" t="n">
-        <v>154</v>
+        <v>19.608</v>
       </c>
       <c r="K3" t="n">
-        <v>1.3319</v>
+        <v>0.1837</v>
       </c>
       <c r="L3" t="n">
-        <v>11716</v>
+        <v>10690.0079</v>
       </c>
       <c r="M3" t="n">
-        <v>13830.5599</v>
+        <v>11703.4798</v>
       </c>
       <c r="N3" t="n">
-        <v>-2114.5599</v>
+        <v>-1013.4718</v>
       </c>
       <c r="O3" t="n">
-        <v>-15.289</v>
+        <v>-8.6595</v>
       </c>
       <c r="P3" t="n">
-        <v>4.2609</v>
+        <v>3.7062</v>
       </c>
       <c r="Q3" t="n">
-        <v>69.1528</v>
+        <v>38.4982</v>
       </c>
       <c r="R3" t="n">
         <v>0</v>
@@ -760,26 +760,26 @@
         <v>0</v>
       </c>
       <c r="V3" t="n">
-        <v>57.81</v>
+        <v>35.1</v>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>https://api.etrade.com/v1/accounts/fOTHyxD-9tctDlNfYkhFzA/portfolio/429040063900.json</t>
+          <t>https://api.etrade.com/v1/accounts/fOTHyxD-9tctDlNfYkhFzA/portfolio/413847387900.json</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>https://api.etrade.com/v1/market/quote/PSTG.json</t>
+          <t>https://api.etrade.com/v1/market/quote/QDTE.json</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>{'symbol': 'PSTG', 'securityType': 'EQ', 'expiryYear': 0, 'expiryMonth': 0, 'expiryDay': 0, 'strikePrice': 0, 'productId': {'symbol': 'PSTG', 'typeCode': 'EQUITY'}}</t>
+          <t>{'symbol': 'QDTE', 'securityType': 'EQ', 'securitySubType': 'ETF', 'expiryYear': 0, 'expiryMonth': 0, 'expiryDay': 0, 'strikePrice': 0, 'productId': {'symbol': 'QDTE', 'typeCode': 'EQUITY'}}</t>
         </is>
       </c>
       <c r="Z3" t="inlineStr">
         <is>
-          <t>{'lastTrade': 58.58, 'lastTradeTime': 1754683800, 'change': 0.77, 'changePct': 1.3319, 'volume': 1771052, 'quoteStatus': 'CLOSING'}</t>
+          <t>{'lastTrade': 35.1645, 'lastTradeTime': 1757527479, 'change': 0.0645, 'changePct': 0.1837, 'volume': 623260, 'quoteStatus': 'REALTIME'}</t>
         </is>
       </c>
       <c r="AA3" t="inlineStr"/>
@@ -819,25 +819,25 @@
         </is>
       </c>
       <c r="J4" t="n">
-        <v>-808</v>
+        <v>-206</v>
       </c>
       <c r="K4" t="n">
-        <v>-10.314</v>
+        <v>-2.8219</v>
       </c>
       <c r="L4" t="n">
-        <v>7026</v>
+        <v>7094</v>
       </c>
       <c r="M4" t="n">
         <v>8757.530000000001</v>
       </c>
       <c r="N4" t="n">
-        <v>-1731.5299</v>
+        <v>-1663.5299</v>
       </c>
       <c r="O4" t="n">
-        <v>-19.7718</v>
+        <v>-18.9954</v>
       </c>
       <c r="P4" t="n">
-        <v>2.5552</v>
+        <v>2.4595</v>
       </c>
       <c r="Q4" t="n">
         <v>43.7876</v>
@@ -855,7 +855,7 @@
         <v>0</v>
       </c>
       <c r="V4" t="n">
-        <v>39.17</v>
+        <v>36.5</v>
       </c>
       <c r="W4" t="inlineStr">
         <is>
@@ -874,7 +874,7 @@
       </c>
       <c r="Z4" t="inlineStr">
         <is>
-          <t>{'lastTrade': 35.13, 'lastTradeTime': 1754683800, 'change': -4.04, 'changePct': -10.314, 'volume': 37478581, 'quoteStatus': 'CLOSING'}</t>
+          <t>{'lastTrade': 35.47, 'lastTradeTime': 1757527585, 'change': -1.03, 'changePct': -2.8219, 'volume': 10155985, 'quoteStatus': 'REALTIME'}</t>
         </is>
       </c>
       <c r="AA4" t="inlineStr"/>
@@ -914,25 +914,25 @@
         </is>
       </c>
       <c r="J5" t="n">
-        <v>13.7599</v>
+        <v>-9.494400000000001</v>
       </c>
       <c r="K5" t="n">
-        <v>0.1036</v>
+        <v>-0.0687</v>
       </c>
       <c r="L5" t="n">
-        <v>13292.1599</v>
+        <v>13798.6656</v>
       </c>
       <c r="M5" t="n">
         <v>13176.0999</v>
       </c>
       <c r="N5" t="n">
-        <v>116.06</v>
+        <v>622.5656</v>
       </c>
       <c r="O5" t="n">
-        <v>0.8808</v>
+        <v>4.7249</v>
       </c>
       <c r="P5" t="n">
-        <v>4.8341</v>
+        <v>4.784</v>
       </c>
       <c r="Q5" t="n">
         <v>19.1513</v>
@@ -950,7 +950,7 @@
         <v>0</v>
       </c>
       <c r="V5" t="n">
-        <v>19.3</v>
+        <v>20.07</v>
       </c>
       <c r="W5" t="inlineStr">
         <is>
@@ -969,7 +969,7 @@
       </c>
       <c r="Z5" t="inlineStr">
         <is>
-          <t>{'lastTrade': 19.32, 'lastTradeTime': 1754683800, 'change': 0.02, 'changePct': 0.1036, 'volume': 2758250, 'quoteStatus': 'CLOSING'}</t>
+          <t>{'lastTrade': 20.0562, 'lastTradeTime': 1757527577, 'change': -0.0138, 'changePct': -0.0687, 'volume': 2069141, 'quoteStatus': 'REALTIME'}</t>
         </is>
       </c>
       <c r="AA5" t="inlineStr"/>
@@ -1009,25 +1009,25 @@
         </is>
       </c>
       <c r="J6" t="n">
-        <v>55.3999</v>
+        <v>83.09990000000001</v>
       </c>
       <c r="K6" t="n">
-        <v>0.4836</v>
+        <v>0.6976</v>
       </c>
       <c r="L6" t="n">
-        <v>11509.35</v>
+        <v>11994.1</v>
       </c>
       <c r="M6" t="n">
         <v>13195.4988</v>
       </c>
       <c r="N6" t="n">
-        <v>-1686.1488</v>
+        <v>-1201.3988</v>
       </c>
       <c r="O6" t="n">
-        <v>-12.7782</v>
+        <v>-9.1046</v>
       </c>
       <c r="P6" t="n">
-        <v>4.1858</v>
+        <v>4.1584</v>
       </c>
       <c r="Q6" t="n">
         <v>9.5274</v>
@@ -1045,7 +1045,7 @@
         <v>0</v>
       </c>
       <c r="V6" t="n">
-        <v>8.27</v>
+        <v>8.6</v>
       </c>
       <c r="W6" t="inlineStr">
         <is>
@@ -1064,7 +1064,7 @@
       </c>
       <c r="Z6" t="inlineStr">
         <is>
-          <t>{'lastTrade': 8.31, 'lastTradeTime': 1754683200, 'change': 0.04, 'changePct': 0.4836, 'volume': 29668, 'quoteStatus': 'CLOSING'}</t>
+          <t>{'lastTrade': 8.66, 'lastTradeTime': 1757527150, 'change': 0.06, 'changePct': 0.6976, 'volume': 19436, 'quoteStatus': 'REALTIME'}</t>
         </is>
       </c>
       <c r="AA6" t="inlineStr"/>
@@ -1104,25 +1104,25 @@
         </is>
       </c>
       <c r="J7" t="n">
-        <v>-13.755</v>
+        <v>11.0039</v>
       </c>
       <c r="K7" t="n">
-        <v>-0.202</v>
+        <v>0.1585</v>
       </c>
       <c r="L7" t="n">
-        <v>6794.97</v>
+        <v>6952.694</v>
       </c>
       <c r="M7" t="n">
         <v>7440.1996</v>
       </c>
       <c r="N7" t="n">
-        <v>-645.2296</v>
+        <v>-487.5056</v>
       </c>
       <c r="O7" t="n">
-        <v>-8.6722</v>
+        <v>-6.5523</v>
       </c>
       <c r="P7" t="n">
-        <v>2.4712</v>
+        <v>2.4105</v>
       </c>
       <c r="Q7" t="n">
         <v>8.1136</v>
@@ -1140,7 +1140,7 @@
         <v>0</v>
       </c>
       <c r="V7" t="n">
-        <v>7.425</v>
+        <v>7.57</v>
       </c>
       <c r="W7" t="inlineStr">
         <is>
@@ -1159,7 +1159,7 @@
       </c>
       <c r="Z7" t="inlineStr">
         <is>
-          <t>{'lastTrade': 7.41, 'lastTradeTime': 1754683800, 'change': -0.015, 'changePct': -0.202, 'volume': 273172, 'quoteStatus': 'CLOSING'}</t>
+          <t>{'lastTrade': 7.582, 'lastTradeTime': 1757526900, 'change': 0.012, 'changePct': 0.1585, 'volume': 74588, 'quoteStatus': 'REALTIME'}</t>
         </is>
       </c>
       <c r="AA7" t="inlineStr"/>
@@ -1199,25 +1199,25 @@
         </is>
       </c>
       <c r="J8" t="n">
-        <v>-47</v>
+        <v>-47.5</v>
       </c>
       <c r="K8" t="n">
-        <v>-1.9207</v>
+        <v>-1.8722</v>
       </c>
       <c r="L8" t="n">
-        <v>2400</v>
+        <v>2489.5</v>
       </c>
       <c r="M8" t="n">
         <v>2620</v>
       </c>
       <c r="N8" t="n">
-        <v>-220</v>
+        <v>-130.5</v>
       </c>
       <c r="O8" t="n">
-        <v>-8.3969</v>
+        <v>-4.9809</v>
       </c>
       <c r="P8" t="n">
-        <v>0.8728</v>
+        <v>0.8631</v>
       </c>
       <c r="Q8" t="n">
         <v>26.2</v>
@@ -1235,7 +1235,7 @@
         <v>0</v>
       </c>
       <c r="V8" t="n">
-        <v>24.47</v>
+        <v>25.37</v>
       </c>
       <c r="W8" t="inlineStr">
         <is>
@@ -1254,25 +1254,25 @@
       </c>
       <c r="Z8" t="inlineStr">
         <is>
-          <t>{'lastTrade': 24.0, 'lastTradeTime': 1754683800, 'change': -0.47, 'changePct': -1.9207, 'volume': 12286726, 'quoteStatus': 'CLOSING'}</t>
+          <t>{'lastTrade': 24.895, 'lastTradeTime': 1757527577, 'change': -0.475, 'changePct': -1.8722, 'volume': 10005056, 'quoteStatus': 'REALTIME'}</t>
         </is>
       </c>
       <c r="AA8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>413847387900</v>
+        <v>454217272900</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>QDTE</t>
+          <t>MRX</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>1732165200000</v>
+        <v>1749009600000</v>
       </c>
       <c r="D9" t="n">
-        <v>38.8379</v>
+        <v>40.6534</v>
       </c>
       <c r="E9" t="n">
         <v>0</v>
@@ -1281,7 +1281,7 @@
         <v>0</v>
       </c>
       <c r="G9" t="n">
-        <v>276</v>
+        <v>300</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
@@ -1294,28 +1294,28 @@
         </is>
       </c>
       <c r="J9" t="n">
-        <v>84.18000000000001</v>
+        <v>-9</v>
       </c>
       <c r="K9" t="n">
-        <v>0.8662</v>
+        <v>-0.0861</v>
       </c>
       <c r="L9" t="n">
-        <v>9802.1399</v>
+        <v>10440</v>
       </c>
       <c r="M9" t="n">
-        <v>10719.2799</v>
+        <v>12196.0398</v>
       </c>
       <c r="N9" t="n">
-        <v>-917.1399</v>
+        <v>-1756.0398</v>
       </c>
       <c r="O9" t="n">
-        <v>-8.555899999999999</v>
+        <v>-14.3984</v>
       </c>
       <c r="P9" t="n">
-        <v>3.5649</v>
+        <v>3.6196</v>
       </c>
       <c r="Q9" t="n">
-        <v>38.8379</v>
+        <v>40.6534</v>
       </c>
       <c r="R9" t="n">
         <v>0</v>
@@ -1330,44 +1330,44 @@
         <v>0</v>
       </c>
       <c r="V9" t="n">
-        <v>35.21</v>
+        <v>34.83</v>
       </c>
       <c r="W9" t="inlineStr">
         <is>
-          <t>https://api.etrade.com/v1/accounts/fOTHyxD-9tctDlNfYkhFzA/portfolio/413847387900.json</t>
+          <t>https://api.etrade.com/v1/accounts/fOTHyxD-9tctDlNfYkhFzA/portfolio/454217272900.json</t>
         </is>
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>https://api.etrade.com/v1/market/quote/QDTE.json</t>
+          <t>https://api.etrade.com/v1/market/quote/MRX.json</t>
         </is>
       </c>
       <c r="Y9" t="inlineStr">
         <is>
-          <t>{'symbol': 'QDTE', 'securityType': 'EQ', 'securitySubType': 'ETF', 'expiryYear': 0, 'expiryMonth': 0, 'expiryDay': 0, 'strikePrice': 0, 'productId': {'symbol': 'QDTE', 'typeCode': 'EQUITY'}}</t>
+          <t>{'symbol': 'MRX', 'securityType': 'EQ', 'expiryYear': 0, 'expiryMonth': 0, 'expiryDay': 0, 'strikePrice': 0, 'productId': {'symbol': 'MRX', 'typeCode': 'EQUITY'}}</t>
         </is>
       </c>
       <c r="Z9" t="inlineStr">
         <is>
-          <t>{'lastTrade': 35.515, 'lastTradeTime': 1754683805, 'change': 0.305, 'changePct': 0.8662, 'volume': 761150, 'quoteStatus': 'CLOSING'}</t>
+          <t>{'lastTrade': 34.8, 'lastTradeTime': 1757527564, 'change': -0.03, 'changePct': -0.0861, 'volume': 241566, 'quoteStatus': 'REALTIME'}</t>
         </is>
       </c>
       <c r="AA9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>372670921900</v>
+        <v>8824507844</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>QYLD</t>
+          <t>QQQI</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>1712030400000</v>
+        <v>1756872000000</v>
       </c>
       <c r="D10" t="n">
-        <v>17.92</v>
+        <v>52.6</v>
       </c>
       <c r="E10" t="n">
         <v>0</v>
@@ -1376,7 +1376,7 @@
         <v>0</v>
       </c>
       <c r="G10" t="n">
-        <v>350</v>
+        <v>110</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
@@ -1389,28 +1389,28 @@
         </is>
       </c>
       <c r="J10" t="n">
-        <v>17.5</v>
+        <v>3.3109</v>
       </c>
       <c r="K10" t="n">
-        <v>0.2969</v>
+        <v>0.0562</v>
       </c>
       <c r="L10" t="n">
-        <v>5911.5</v>
+        <v>5889.411</v>
       </c>
       <c r="M10" t="n">
-        <v>6272</v>
+        <v>5786</v>
       </c>
       <c r="N10" t="n">
-        <v>-360.5</v>
+        <v>103.411</v>
       </c>
       <c r="O10" t="n">
-        <v>-5.7477</v>
+        <v>1.7872</v>
       </c>
       <c r="P10" t="n">
-        <v>2.1499</v>
+        <v>2.0418</v>
       </c>
       <c r="Q10" t="n">
-        <v>17.92</v>
+        <v>52.6</v>
       </c>
       <c r="R10" t="n">
         <v>0</v>
@@ -1425,44 +1425,44 @@
         <v>0</v>
       </c>
       <c r="V10" t="n">
-        <v>16.84</v>
+        <v>53.51</v>
       </c>
       <c r="W10" t="inlineStr">
         <is>
-          <t>https://api.etrade.com/v1/accounts/fOTHyxD-9tctDlNfYkhFzA/portfolio/372670921900.json</t>
+          <t>https://api.etrade.com/v1/accounts/fOTHyxD-9tctDlNfYkhFzA/portfolio/8824507844.json</t>
         </is>
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>https://api.etrade.com/v1/market/quote/QYLD.json</t>
+          <t>https://api.etrade.com/v1/market/quote/QQQI.json</t>
         </is>
       </c>
       <c r="Y10" t="inlineStr">
         <is>
-          <t>{'symbol': 'QYLD', 'securityType': 'EQ', 'securitySubType': 'ETF', 'expiryYear': 0, 'expiryMonth': 0, 'expiryDay': 0, 'strikePrice': 0, 'productId': {'symbol': 'QYLD', 'typeCode': 'EQUITY'}}</t>
+          <t>{'symbol': 'QQQI', 'securityType': 'EQ', 'securitySubType': 'ETF', 'expiryYear': 0, 'expiryMonth': 0, 'expiryDay': 0, 'strikePrice': 0, 'productId': {'symbol': 'QQQI', 'typeCode': 'EQUITY'}}</t>
         </is>
       </c>
       <c r="Z10" t="inlineStr">
         <is>
-          <t>{'lastTrade': 16.89, 'lastTradeTime': 1754684100, 'change': 0.05, 'changePct': 0.2969, 'volume': 2870871, 'quoteStatus': 'CLOSING'}</t>
+          <t>{'lastTrade': 53.5401, 'lastTradeTime': 1757527582, 'change': 0.0301, 'changePct': 0.0562, 'volume': 2833413, 'quoteStatus': 'REALTIME'}</t>
         </is>
       </c>
       <c r="AA10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>387090035900</v>
+        <v>372291315900</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>SOXL</t>
+          <t>RYLD</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>1719374400000</v>
+        <v>1711944000000</v>
       </c>
       <c r="D11" t="n">
-        <v>54.4218</v>
+        <v>16.5407</v>
       </c>
       <c r="E11" t="n">
         <v>0</v>
@@ -1471,7 +1471,7 @@
         <v>0</v>
       </c>
       <c r="G11" t="n">
-        <v>110</v>
+        <v>579</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
@@ -1484,28 +1484,28 @@
         </is>
       </c>
       <c r="J11" t="n">
-        <v>78.09990000000001</v>
+        <v>2.0264</v>
       </c>
       <c r="K11" t="n">
-        <v>2.8399</v>
+        <v>0.023</v>
       </c>
       <c r="L11" t="n">
-        <v>2828.0999</v>
+        <v>8808.6165</v>
       </c>
       <c r="M11" t="n">
-        <v>5986.3999</v>
+        <v>9577.069299999999</v>
       </c>
       <c r="N11" t="n">
-        <v>-3158.2999</v>
+        <v>-768.4528</v>
       </c>
       <c r="O11" t="n">
-        <v>-52.7579</v>
+        <v>-8.0238</v>
       </c>
       <c r="P11" t="n">
-        <v>1.0285</v>
+        <v>3.0539</v>
       </c>
       <c r="Q11" t="n">
-        <v>54.4218</v>
+        <v>16.5407</v>
       </c>
       <c r="R11" t="n">
         <v>0</v>
@@ -1520,53 +1520,53 @@
         <v>0</v>
       </c>
       <c r="V11" t="n">
-        <v>25</v>
+        <v>15.21</v>
       </c>
       <c r="W11" t="inlineStr">
         <is>
-          <t>https://api.etrade.com/v1/accounts/fOTHyxD-9tctDlNfYkhFzA/portfolio/387090035900.json</t>
+          <t>https://api.etrade.com/v1/accounts/fOTHyxD-9tctDlNfYkhFzA/portfolio/372291315900.json</t>
         </is>
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>https://api.etrade.com/v1/market/quote/SOXL.json</t>
+          <t>https://api.etrade.com/v1/market/quote/RYLD.json</t>
         </is>
       </c>
       <c r="Y11" t="inlineStr">
         <is>
-          <t>{'symbol': 'SOXL', 'securityType': 'EQ', 'securitySubType': 'ETF', 'expiryYear': 0, 'expiryMonth': 0, 'expiryDay': 0, 'strikePrice': 0, 'productId': {'symbol': 'SOXL', 'typeCode': 'EQUITY'}}</t>
+          <t>{'symbol': 'RYLD', 'securityType': 'EQ', 'securitySubType': 'ETF', 'expiryYear': 0, 'expiryMonth': 0, 'expiryDay': 0, 'strikePrice': 0, 'productId': {'symbol': 'RYLD', 'typeCode': 'EQUITY'}}</t>
         </is>
       </c>
       <c r="Z11" t="inlineStr">
         <is>
-          <t>{'lastTrade': 25.71, 'lastTradeTime': 1754683800, 'change': 0.71, 'changePct': 2.84, 'volume': 71389885, 'quoteStatus': 'CLOSING'}</t>
+          <t>{'lastTrade': 15.2135, 'lastTradeTime': 1757527560, 'change': 0.0035, 'changePct': 0.023, 'volume': 347721, 'quoteStatus': 'REALTIME'}</t>
         </is>
       </c>
       <c r="AA11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>899082844</v>
+        <v>465023009900</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>SOFI Sep 19 '25 $27 Put</t>
+          <t>SMCI</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>1753848000000</v>
+        <v>1753243200000</v>
       </c>
       <c r="D12" t="n">
-        <v>6</v>
+        <v>50.4275</v>
       </c>
       <c r="E12" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F12" t="n">
-        <v>0.08</v>
+        <v>0</v>
       </c>
       <c r="G12" t="n">
-        <v>-4</v>
+        <v>400</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
@@ -1575,32 +1575,32 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>SHORT</t>
+          <t>LONG</t>
         </is>
       </c>
       <c r="J12" t="n">
-        <v>0</v>
+        <v>400</v>
       </c>
       <c r="K12" t="n">
-        <v>0</v>
+        <v>2.3299</v>
       </c>
       <c r="L12" t="n">
-        <v>-2060</v>
+        <v>17568</v>
       </c>
       <c r="M12" t="n">
-        <v>-2397.92</v>
+        <v>20171.04</v>
       </c>
       <c r="N12" t="n">
-        <v>337.92</v>
+        <v>-2603.0399</v>
       </c>
       <c r="O12" t="n">
-        <v>14.0922</v>
+        <v>-12.9048</v>
       </c>
       <c r="P12" t="n">
-        <v>-0.7491</v>
+        <v>6.0909</v>
       </c>
       <c r="Q12" t="n">
-        <v>5.9948</v>
+        <v>50.4276</v>
       </c>
       <c r="R12" t="n">
         <v>0</v>
@@ -1615,48 +1615,44 @@
         <v>0</v>
       </c>
       <c r="V12" t="n">
-        <v>5.15</v>
+        <v>42.92</v>
       </c>
       <c r="W12" t="inlineStr">
         <is>
-          <t>https://api.etrade.com/v1/accounts/fOTHyxD-9tctDlNfYkhFzA/portfolio/899082844.json</t>
+          <t>https://api.etrade.com/v1/accounts/fOTHyxD-9tctDlNfYkhFzA/portfolio/465023009900.json</t>
         </is>
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>https://api.etrade.com/v1/market/quote/SOFI:2025:9:19:PUT:27.json</t>
+          <t>https://api.etrade.com/v1/market/quote/SMCI.json</t>
         </is>
       </c>
       <c r="Y12" t="inlineStr">
         <is>
-          <t>{'symbol': 'SOFI', 'securityType': 'OPTN', 'callPut': 'PUT', 'expiryYear': 2025, 'expiryMonth': 9, 'expiryDay': 19, 'strikePrice': 27, 'productId': {'symbol': 'SOFI', 'typeCode': 'EQUITY'}}</t>
+          <t>{'symbol': 'SMCI', 'securityType': 'EQ', 'expiryYear': 0, 'expiryMonth': 0, 'expiryDay': 0, 'strikePrice': 0, 'productId': {'symbol': 'SMCI', 'typeCode': 'EQUITY'}}</t>
         </is>
       </c>
       <c r="Z12" t="inlineStr">
         <is>
-          <t>{'lastTrade': 5.15, 'lastTradeTime': 1754683195, 'change': 0, 'changePct': 0, 'volume': 0, 'quoteStatus': 'REALTIME'}</t>
-        </is>
-      </c>
-      <c r="AA12" t="inlineStr">
-        <is>
-          <t>SOFI--250919P00027000</t>
-        </is>
-      </c>
+          <t>{'lastTrade': 43.92, 'lastTradeTime': 1757527586, 'change': 1, 'changePct': 2.3299, 'volume': 30736392, 'quoteStatus': 'REALTIME'}</t>
+        </is>
+      </c>
+      <c r="AA12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>906376844</v>
+        <v>4592870844</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>SOFI</t>
+          <t>UGL</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1753848000000</v>
+        <v>1755144000000</v>
       </c>
       <c r="D13" t="n">
-        <v>21.6999</v>
+        <v>35.1</v>
       </c>
       <c r="E13" t="n">
         <v>0</v>
@@ -1665,7 +1661,7 @@
         <v>0</v>
       </c>
       <c r="G13" t="n">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
@@ -1678,28 +1674,28 @@
         </is>
       </c>
       <c r="J13" t="n">
-        <v>4</v>
+        <v>42</v>
       </c>
       <c r="K13" t="n">
-        <v>0.0905</v>
+        <v>1.0241</v>
       </c>
       <c r="L13" t="n">
-        <v>4420</v>
+        <v>4143</v>
       </c>
       <c r="M13" t="n">
-        <v>4340</v>
+        <v>3510</v>
       </c>
       <c r="N13" t="n">
-        <v>80</v>
+        <v>633</v>
       </c>
       <c r="O13" t="n">
-        <v>1.8433</v>
+        <v>18.0341</v>
       </c>
       <c r="P13" t="n">
-        <v>1.6074</v>
+        <v>1.4364</v>
       </c>
       <c r="Q13" t="n">
-        <v>21.7</v>
+        <v>35.1</v>
       </c>
       <c r="R13" t="n">
         <v>0</v>
@@ -1714,53 +1710,53 @@
         <v>0</v>
       </c>
       <c r="V13" t="n">
-        <v>22.08</v>
+        <v>41.01</v>
       </c>
       <c r="W13" t="inlineStr">
         <is>
-          <t>https://api.etrade.com/v1/accounts/fOTHyxD-9tctDlNfYkhFzA/portfolio/906376844.json</t>
+          <t>https://api.etrade.com/v1/accounts/fOTHyxD-9tctDlNfYkhFzA/portfolio/4592870844.json</t>
         </is>
       </c>
       <c r="X13" t="inlineStr">
         <is>
-          <t>https://api.etrade.com/v1/market/quote/SOFI.json</t>
+          <t>https://api.etrade.com/v1/market/quote/UGL.json</t>
         </is>
       </c>
       <c r="Y13" t="inlineStr">
         <is>
-          <t>{'symbol': 'SOFI', 'securityType': 'EQ', 'expiryYear': 0, 'expiryMonth': 0, 'expiryDay': 0, 'strikePrice': 0, 'productId': {'symbol': 'SOFI', 'typeCode': 'EQUITY'}}</t>
+          <t>{'symbol': 'UGL', 'securityType': 'EQ', 'securitySubType': 'ETF', 'expiryYear': 0, 'expiryMonth': 0, 'expiryDay': 0, 'strikePrice': 0, 'productId': {'symbol': 'UGL', 'typeCode': 'EQUITY'}}</t>
         </is>
       </c>
       <c r="Z13" t="inlineStr">
         <is>
-          <t>{'lastTrade': 22.1, 'lastTradeTime': 1754683200, 'change': 0.02, 'changePct': 0.0905, 'volume': 49146091, 'quoteStatus': 'CLOSING'}</t>
+          <t>{'lastTrade': 41.43, 'lastTradeTime': 1757527507, 'change': 0.42, 'changePct': 1.0241, 'volume': 1168665, 'quoteStatus': 'REALTIME'}</t>
         </is>
       </c>
       <c r="AA13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>465007953900</v>
+        <v>385208533900</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>SMCI Sep 19 '25 $60 Put</t>
+          <t>SVOL</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>1753243200000</v>
+        <v>1718337600000</v>
       </c>
       <c r="D14" t="n">
-        <v>10.9</v>
+        <v>22.3287</v>
       </c>
       <c r="E14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F14" t="n">
-        <v>0.04</v>
+        <v>0</v>
       </c>
       <c r="G14" t="n">
-        <v>-2</v>
+        <v>552</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
@@ -1769,32 +1765,32 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>SHORT</t>
+          <t>LONG</t>
         </is>
       </c>
       <c r="J14" t="n">
-        <v>0</v>
+        <v>22.0799</v>
       </c>
       <c r="K14" t="n">
-        <v>0</v>
+        <v>0.2247</v>
       </c>
       <c r="L14" t="n">
-        <v>-3175</v>
+        <v>9847.68</v>
       </c>
       <c r="M14" t="n">
-        <v>-2178.96</v>
+        <v>12325.4898</v>
       </c>
       <c r="N14" t="n">
-        <v>-996.0399</v>
+        <v>-2477.8098</v>
       </c>
       <c r="O14" t="n">
-        <v>-45.7117</v>
+        <v>-20.1031</v>
       </c>
       <c r="P14" t="n">
-        <v>-1.1547</v>
+        <v>3.4142</v>
       </c>
       <c r="Q14" t="n">
-        <v>10.8948</v>
+        <v>22.3287</v>
       </c>
       <c r="R14" t="n">
         <v>0</v>
@@ -1809,48 +1805,44 @@
         <v>0</v>
       </c>
       <c r="V14" t="n">
-        <v>15.875</v>
+        <v>17.8</v>
       </c>
       <c r="W14" t="inlineStr">
         <is>
-          <t>https://api.etrade.com/v1/accounts/fOTHyxD-9tctDlNfYkhFzA/portfolio/465007953900.json</t>
+          <t>https://api.etrade.com/v1/accounts/fOTHyxD-9tctDlNfYkhFzA/portfolio/385208533900.json</t>
         </is>
       </c>
       <c r="X14" t="inlineStr">
         <is>
-          <t>https://api.etrade.com/v1/market/quote/SMCI:2025:9:19:PUT:60.json</t>
+          <t>https://api.etrade.com/v1/market/quote/SVOL.json</t>
         </is>
       </c>
       <c r="Y14" t="inlineStr">
         <is>
-          <t>{'symbol': 'SMCI', 'securityType': 'OPTN', 'callPut': 'PUT', 'expiryYear': 2025, 'expiryMonth': 9, 'expiryDay': 19, 'strikePrice': 60, 'productId': {'symbol': 'SMCI', 'typeCode': 'EQUITY'}}</t>
+          <t>{'symbol': 'SVOL', 'securityType': 'EQ', 'securitySubType': 'ETF', 'expiryYear': 0, 'expiryMonth': 0, 'expiryDay': 0, 'strikePrice': 0, 'productId': {'symbol': 'SVOL', 'typeCode': 'EQUITY'}}</t>
         </is>
       </c>
       <c r="Z14" t="inlineStr">
         <is>
-          <t>{'lastTrade': 15.75, 'lastTradeTime': 1754683199, 'change': 0, 'changePct': 0, 'volume': 56, 'quoteStatus': 'REALTIME'}</t>
-        </is>
-      </c>
-      <c r="AA14" t="inlineStr">
-        <is>
-          <t>SMCI--250919P00060000</t>
-        </is>
-      </c>
+          <t>{'lastTrade': 17.84, 'lastTradeTime': 1757527466, 'change': 0.04, 'changePct': 0.2247, 'volume': 188412, 'quoteStatus': 'REALTIME'}</t>
+        </is>
+      </c>
+      <c r="AA14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>465023009900</v>
+        <v>387090035900</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>SMCI</t>
+          <t>SOXL</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>1753243200000</v>
+        <v>1719374400000</v>
       </c>
       <c r="D15" t="n">
-        <v>51.75</v>
+        <v>54.4218</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
@@ -1859,7 +1851,7 @@
         <v>0</v>
       </c>
       <c r="G15" t="n">
-        <v>200</v>
+        <v>110</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
@@ -1872,28 +1864,28 @@
         </is>
       </c>
       <c r="J15" t="n">
-        <v>-414</v>
+        <v>135.3</v>
       </c>
       <c r="K15" t="n">
-        <v>-4.4353</v>
+        <v>4.5253</v>
       </c>
       <c r="L15" t="n">
-        <v>8920</v>
+        <v>3125.0999</v>
       </c>
       <c r="M15" t="n">
-        <v>10350</v>
+        <v>5986.3999</v>
       </c>
       <c r="N15" t="n">
-        <v>-1430</v>
+        <v>-2861.2999</v>
       </c>
       <c r="O15" t="n">
-        <v>-13.8164</v>
+        <v>-47.7966</v>
       </c>
       <c r="P15" t="n">
-        <v>3.244</v>
+        <v>1.0834</v>
       </c>
       <c r="Q15" t="n">
-        <v>51.75</v>
+        <v>54.4218</v>
       </c>
       <c r="R15" t="n">
         <v>0</v>
@@ -1908,53 +1900,53 @@
         <v>0</v>
       </c>
       <c r="V15" t="n">
-        <v>46.67</v>
+        <v>27.18</v>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>https://api.etrade.com/v1/accounts/fOTHyxD-9tctDlNfYkhFzA/portfolio/465023009900.json</t>
+          <t>https://api.etrade.com/v1/accounts/fOTHyxD-9tctDlNfYkhFzA/portfolio/387090035900.json</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>https://api.etrade.com/v1/market/quote/SMCI.json</t>
+          <t>https://api.etrade.com/v1/market/quote/SOXL.json</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
-          <t>{'symbol': 'SMCI', 'securityType': 'EQ', 'expiryYear': 0, 'expiryMonth': 0, 'expiryDay': 0, 'strikePrice': 0, 'productId': {'symbol': 'SMCI', 'typeCode': 'EQUITY'}}</t>
+          <t>{'symbol': 'SOXL', 'securityType': 'EQ', 'securitySubType': 'ETF', 'expiryYear': 0, 'expiryMonth': 0, 'expiryDay': 0, 'strikePrice': 0, 'productId': {'symbol': 'SOXL', 'typeCode': 'EQUITY'}}</t>
         </is>
       </c>
       <c r="Z15" t="inlineStr">
         <is>
-          <t>{'lastTrade': 44.6, 'lastTradeTime': 1754683200, 'change': -2.07, 'changePct': -4.4353, 'volume': 43796793, 'quoteStatus': 'CLOSING'}</t>
+          <t>{'lastTrade': 28.41, 'lastTradeTime': 1757527586, 'change': 1.23, 'changePct': 4.5253, 'volume': 63076365, 'quoteStatus': 'REALTIME'}</t>
         </is>
       </c>
       <c r="AA15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>372291315900</v>
+        <v>8114240844</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>RYLD</t>
+          <t>SOUN Oct 17 '25 $17 Put</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>1711944000000</v>
+        <v>1756440000000</v>
       </c>
       <c r="D16" t="n">
-        <v>16.5407</v>
+        <v>5</v>
       </c>
       <c r="E16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F16" t="n">
-        <v>0</v>
+        <v>0.04</v>
       </c>
       <c r="G16" t="n">
-        <v>579</v>
+        <v>-2</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
@@ -1963,32 +1955,32 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>LONG</t>
+          <t>SHORT</t>
         </is>
       </c>
       <c r="J16" t="n">
-        <v>23.16</v>
+        <v>-85</v>
       </c>
       <c r="K16" t="n">
-        <v>0.271</v>
+        <v>-13.7096</v>
       </c>
       <c r="L16" t="n">
-        <v>8569.200000000001</v>
+        <v>-705</v>
       </c>
       <c r="M16" t="n">
-        <v>9577.069299999999</v>
+        <v>-998.96</v>
       </c>
       <c r="N16" t="n">
-        <v>-1007.8693</v>
+        <v>293.9599</v>
       </c>
       <c r="O16" t="n">
-        <v>-10.5237</v>
+        <v>29.4266</v>
       </c>
       <c r="P16" t="n">
-        <v>3.1165</v>
+        <v>-0.2444</v>
       </c>
       <c r="Q16" t="n">
-        <v>16.5407</v>
+        <v>4.9948</v>
       </c>
       <c r="R16" t="n">
         <v>0</v>
@@ -2003,53 +1995,57 @@
         <v>0</v>
       </c>
       <c r="V16" t="n">
-        <v>14.76</v>
+        <v>3.1</v>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>https://api.etrade.com/v1/accounts/fOTHyxD-9tctDlNfYkhFzA/portfolio/372291315900.json</t>
+          <t>https://api.etrade.com/v1/accounts/fOTHyxD-9tctDlNfYkhFzA/portfolio/8114240844.json</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>https://api.etrade.com/v1/market/quote/RYLD.json</t>
+          <t>https://api.etrade.com/v1/market/quote/SOUN:2025:10:17:PUT:17.json</t>
         </is>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>{'symbol': 'RYLD', 'securityType': 'EQ', 'securitySubType': 'ETF', 'expiryYear': 0, 'expiryMonth': 0, 'expiryDay': 0, 'strikePrice': 0, 'productId': {'symbol': 'RYLD', 'typeCode': 'EQUITY'}}</t>
+          <t>{'symbol': 'SOUN', 'securityType': 'OPTN', 'callPut': 'PUT', 'expiryYear': 2025, 'expiryMonth': 10, 'expiryDay': 17, 'strikePrice': 17, 'productId': {'symbol': 'SOUN', 'typeCode': 'EQUITY'}}</t>
         </is>
       </c>
       <c r="Z16" t="inlineStr">
         <is>
-          <t>{'lastTrade': 14.8, 'lastTradeTime': 1754683800, 'change': 0.04, 'changePct': 0.271, 'volume': 495676, 'quoteStatus': 'CLOSING'}</t>
-        </is>
-      </c>
-      <c r="AA16" t="inlineStr"/>
+          <t>{'lastTrade': 3.45, 'lastTradeTime': 1757527580, 'change': 0.425, 'changePct': 13.7096, 'volume': 22, 'quoteStatus': 'REALTIME'}</t>
+        </is>
+      </c>
+      <c r="AA16" t="inlineStr">
+        <is>
+          <t>SOUN--251017P00017000</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>454217272900</v>
+        <v>9016754844</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>MRX</t>
+          <t>SOFI Oct 17 '25 $28 Put</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>1749009600000</v>
+        <v>1756872000000</v>
       </c>
       <c r="D17" t="n">
-        <v>40.6534</v>
+        <v>4.15</v>
       </c>
       <c r="E17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F17" t="n">
-        <v>0</v>
+        <v>0.04</v>
       </c>
       <c r="G17" t="n">
-        <v>300</v>
+        <v>-2</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
@@ -2058,32 +2054,32 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>LONG</t>
+          <t>SHORT</t>
         </is>
       </c>
       <c r="J17" t="n">
-        <v>-33</v>
+        <v>-50</v>
       </c>
       <c r="K17" t="n">
-        <v>-0.3096</v>
+        <v>-8.064500000000001</v>
       </c>
       <c r="L17" t="n">
-        <v>10623</v>
+        <v>-670</v>
       </c>
       <c r="M17" t="n">
-        <v>12196.0398</v>
+        <v>-828.96</v>
       </c>
       <c r="N17" t="n">
-        <v>-1573.0398</v>
+        <v>158.96</v>
       </c>
       <c r="O17" t="n">
-        <v>-12.8979</v>
+        <v>19.1758</v>
       </c>
       <c r="P17" t="n">
-        <v>3.8634</v>
+        <v>-0.2322</v>
       </c>
       <c r="Q17" t="n">
-        <v>40.6534</v>
+        <v>4.1448</v>
       </c>
       <c r="R17" t="n">
         <v>0</v>
@@ -2098,53 +2094,57 @@
         <v>0</v>
       </c>
       <c r="V17" t="n">
-        <v>35.52</v>
+        <v>3.1</v>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>https://api.etrade.com/v1/accounts/fOTHyxD-9tctDlNfYkhFzA/portfolio/454217272900.json</t>
+          <t>https://api.etrade.com/v1/accounts/fOTHyxD-9tctDlNfYkhFzA/portfolio/9016754844.json</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>https://api.etrade.com/v1/market/quote/MRX.json</t>
+          <t>https://api.etrade.com/v1/market/quote/SOFI:2025:10:17:PUT:28.json</t>
         </is>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>{'symbol': 'MRX', 'securityType': 'EQ', 'expiryYear': 0, 'expiryMonth': 0, 'expiryDay': 0, 'strikePrice': 0, 'productId': {'symbol': 'MRX', 'typeCode': 'EQUITY'}}</t>
+          <t>{'symbol': 'SOFI', 'securityType': 'OPTN', 'callPut': 'PUT', 'expiryYear': 2025, 'expiryMonth': 10, 'expiryDay': 17, 'strikePrice': 28, 'productId': {'symbol': 'SOFI', 'typeCode': 'EQUITY'}}</t>
         </is>
       </c>
       <c r="Z17" t="inlineStr">
         <is>
-          <t>{'lastTrade': 35.41, 'lastTradeTime': 1754683200, 'change': -0.11, 'changePct': -0.3096, 'volume': 1146213, 'quoteStatus': 'CLOSING'}</t>
-        </is>
-      </c>
-      <c r="AA17" t="inlineStr"/>
+          <t>{'lastTrade': 3.35, 'lastTradeTime': 1757527576, 'change': 0.25, 'changePct': 8.0645, 'volume': 34, 'quoteStatus': 'REALTIME'}</t>
+        </is>
+      </c>
+      <c r="AA17" t="inlineStr">
+        <is>
+          <t>SOFI--251017P00028000</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>439396792900</v>
+        <v>6895407844</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>MORT</t>
+          <t>SOFI Sep 19 '25 $27 Call</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>1742961600000</v>
+        <v>1756094400000</v>
       </c>
       <c r="D18" t="n">
-        <v>11.3</v>
+        <v>1</v>
       </c>
       <c r="E18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F18" t="n">
-        <v>0</v>
+        <v>0.04</v>
       </c>
       <c r="G18" t="n">
-        <v>90</v>
+        <v>-2</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
@@ -2153,32 +2153,32 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>LONG</t>
+          <t>SHORT</t>
         </is>
       </c>
       <c r="J18" t="n">
-        <v>1.8</v>
+        <v>29</v>
       </c>
       <c r="K18" t="n">
-        <v>0.1888</v>
+        <v>23.7704</v>
       </c>
       <c r="L18" t="n">
-        <v>954.8999</v>
+        <v>-93</v>
       </c>
       <c r="M18" t="n">
-        <v>1017</v>
+        <v>-198.96</v>
       </c>
       <c r="N18" t="n">
-        <v>-62.1</v>
+        <v>105.9599</v>
       </c>
       <c r="O18" t="n">
-        <v>-6.1061</v>
+        <v>53.2569</v>
       </c>
       <c r="P18" t="n">
-        <v>0.3472</v>
+        <v>-0.0322</v>
       </c>
       <c r="Q18" t="n">
-        <v>11.3</v>
+        <v>0.9948</v>
       </c>
       <c r="R18" t="n">
         <v>0</v>
@@ -2193,44 +2193,48 @@
         <v>0</v>
       </c>
       <c r="V18" t="n">
-        <v>10.59</v>
+        <v>0.61</v>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>https://api.etrade.com/v1/accounts/fOTHyxD-9tctDlNfYkhFzA/portfolio/439396792900.json</t>
+          <t>https://api.etrade.com/v1/accounts/fOTHyxD-9tctDlNfYkhFzA/portfolio/6895407844.json</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>https://api.etrade.com/v1/market/quote/MORT.json</t>
+          <t>https://api.etrade.com/v1/market/quote/SOFI:2025:9:19:CALL:27.json</t>
         </is>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>{'symbol': 'MORT', 'securityType': 'EQ', 'securitySubType': 'ETF', 'expiryYear': 0, 'expiryMonth': 0, 'expiryDay': 0, 'strikePrice': 0, 'productId': {'symbol': 'MORT', 'typeCode': 'EQUITY'}}</t>
+          <t>{'symbol': 'SOFI', 'securityType': 'OPTN', 'callPut': 'CALL', 'expiryYear': 2025, 'expiryMonth': 9, 'expiryDay': 19, 'strikePrice': 27, 'productId': {'symbol': 'SOFI', 'typeCode': 'EQUITY'}}</t>
         </is>
       </c>
       <c r="Z18" t="inlineStr">
         <is>
-          <t>{'lastTrade': 10.61, 'lastTradeTime': 1754683800, 'change': 0.02, 'changePct': 0.1888, 'volume': 269870, 'quoteStatus': 'CLOSING'}</t>
-        </is>
-      </c>
-      <c r="AA18" t="inlineStr"/>
+          <t>{'lastTrade': 0.47, 'lastTradeTime': 1757527582, 'change': -0.145, 'changePct': -23.7704, 'volume': 5264, 'quoteStatus': 'REALTIME'}</t>
+        </is>
+      </c>
+      <c r="AA18" t="inlineStr">
+        <is>
+          <t>SOFI--250919C00027000</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>415421866900</v>
+        <v>906376844</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>MARA</t>
+          <t>SOFI</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>1733115600000</v>
+        <v>1753848000000</v>
       </c>
       <c r="D19" t="n">
-        <v>22.8027</v>
+        <v>21.6999</v>
       </c>
       <c r="E19" t="n">
         <v>0</v>
@@ -2239,7 +2243,7 @@
         <v>0</v>
       </c>
       <c r="G19" t="n">
-        <v>400</v>
+        <v>200</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
@@ -2252,28 +2256,28 @@
         </is>
       </c>
       <c r="J19" t="n">
-        <v>-228</v>
+        <v>-82.8599</v>
       </c>
       <c r="K19" t="n">
-        <v>-3.5736</v>
+        <v>-1.5953</v>
       </c>
       <c r="L19" t="n">
-        <v>6152</v>
+        <v>5111.14</v>
       </c>
       <c r="M19" t="n">
-        <v>9121.110000000001</v>
+        <v>4340</v>
       </c>
       <c r="N19" t="n">
-        <v>-2969.11</v>
+        <v>771.1399</v>
       </c>
       <c r="O19" t="n">
-        <v>-32.552</v>
+        <v>17.7682</v>
       </c>
       <c r="P19" t="n">
-        <v>2.2374</v>
+        <v>1.772</v>
       </c>
       <c r="Q19" t="n">
-        <v>22.8027</v>
+        <v>21.7</v>
       </c>
       <c r="R19" t="n">
         <v>0</v>
@@ -2288,44 +2292,44 @@
         <v>0</v>
       </c>
       <c r="V19" t="n">
-        <v>15.95</v>
+        <v>25.97</v>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>https://api.etrade.com/v1/accounts/fOTHyxD-9tctDlNfYkhFzA/portfolio/415421866900.json</t>
+          <t>https://api.etrade.com/v1/accounts/fOTHyxD-9tctDlNfYkhFzA/portfolio/906376844.json</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>https://api.etrade.com/v1/market/quote/MARA.json</t>
+          <t>https://api.etrade.com/v1/market/quote/SOFI.json</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
-          <t>{'symbol': 'MARA', 'securityType': 'EQ', 'expiryYear': 0, 'expiryMonth': 0, 'expiryDay': 0, 'strikePrice': 0, 'productId': {'symbol': 'MARA', 'typeCode': 'EQUITY'}}</t>
+          <t>{'symbol': 'SOFI', 'securityType': 'EQ', 'expiryYear': 0, 'expiryMonth': 0, 'expiryDay': 0, 'strikePrice': 0, 'productId': {'symbol': 'SOFI', 'typeCode': 'EQUITY'}}</t>
         </is>
       </c>
       <c r="Z19" t="inlineStr">
         <is>
-          <t>{'lastTrade': 15.38, 'lastTradeTime': 1754683200, 'change': -0.57, 'changePct': -3.5736, 'volume': 25638852, 'quoteStatus': 'CLOSING'}</t>
+          <t>{'lastTrade': 25.5557, 'lastTradeTime': 1757527586, 'change': -0.4143, 'changePct': -1.5953, 'volume': 45648910, 'quoteStatus': 'REALTIME'}</t>
         </is>
       </c>
       <c r="AA19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>374009142900</v>
+        <v>439396792900</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>CHMI</t>
+          <t>MORT</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>1712635200000</v>
+        <v>1742961600000</v>
       </c>
       <c r="D20" t="n">
-        <v>3.3992</v>
+        <v>11.3</v>
       </c>
       <c r="E20" t="n">
         <v>0</v>
@@ -2334,7 +2338,7 @@
         <v>0</v>
       </c>
       <c r="G20" t="n">
-        <v>2425</v>
+        <v>90</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
@@ -2347,28 +2351,28 @@
         </is>
       </c>
       <c r="J20" t="n">
-        <v>145.5</v>
+        <v>-4.5</v>
       </c>
       <c r="K20" t="n">
-        <v>2.1505</v>
+        <v>-0.4436</v>
       </c>
       <c r="L20" t="n">
-        <v>6911.25</v>
+        <v>1009.7999</v>
       </c>
       <c r="M20" t="n">
-        <v>8243.249100000001</v>
+        <v>1017</v>
       </c>
       <c r="N20" t="n">
-        <v>-1331.9991</v>
+        <v>-7.2</v>
       </c>
       <c r="O20" t="n">
-        <v>-16.1586</v>
+        <v>-0.7079</v>
       </c>
       <c r="P20" t="n">
-        <v>2.5135</v>
+        <v>0.3501</v>
       </c>
       <c r="Q20" t="n">
-        <v>3.3992</v>
+        <v>11.3</v>
       </c>
       <c r="R20" t="n">
         <v>0</v>
@@ -2383,44 +2387,44 @@
         <v>0</v>
       </c>
       <c r="V20" t="n">
-        <v>2.79</v>
+        <v>11.27</v>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>https://api.etrade.com/v1/accounts/fOTHyxD-9tctDlNfYkhFzA/portfolio/374009142900.json</t>
+          <t>https://api.etrade.com/v1/accounts/fOTHyxD-9tctDlNfYkhFzA/portfolio/439396792900.json</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>https://api.etrade.com/v1/market/quote/CHMI.json</t>
+          <t>https://api.etrade.com/v1/market/quote/MORT.json</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>{'symbol': 'CHMI', 'securityType': 'EQ', 'expiryYear': 0, 'expiryMonth': 0, 'expiryDay': 0, 'strikePrice': 0, 'productId': {'symbol': 'CHMI', 'typeCode': 'EQUITY'}}</t>
+          <t>{'symbol': 'MORT', 'securityType': 'EQ', 'securitySubType': 'ETF', 'expiryYear': 0, 'expiryMonth': 0, 'expiryDay': 0, 'strikePrice': 0, 'productId': {'symbol': 'MORT', 'typeCode': 'EQUITY'}}</t>
         </is>
       </c>
       <c r="Z20" t="inlineStr">
         <is>
-          <t>{'lastTrade': 2.85, 'lastTradeTime': 1754683800, 'change': 0.06, 'changePct': 2.1505, 'volume': 295290, 'quoteStatus': 'CLOSING'}</t>
+          <t>{'lastTrade': 11.22, 'lastTradeTime': 1757527486, 'change': -0.05, 'changePct': -0.4436, 'volume': 521991, 'quoteStatus': 'REALTIME'}</t>
         </is>
       </c>
       <c r="AA20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>387800975900</v>
+        <v>415421866900</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>BRSP</t>
+          <t>MARA</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>1719806400000</v>
+        <v>1733115600000</v>
       </c>
       <c r="D21" t="n">
-        <v>5.7</v>
+        <v>22.8027</v>
       </c>
       <c r="E21" t="n">
         <v>0</v>
@@ -2429,7 +2433,7 @@
         <v>0</v>
       </c>
       <c r="G21" t="n">
-        <v>568</v>
+        <v>400</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
@@ -2442,28 +2446,28 @@
         </is>
       </c>
       <c r="J21" t="n">
-        <v>-5.6799</v>
+        <v>63.96</v>
       </c>
       <c r="K21" t="n">
-        <v>-0.1872</v>
+        <v>1.0037</v>
       </c>
       <c r="L21" t="n">
-        <v>3027.44</v>
+        <v>6435.96</v>
       </c>
       <c r="M21" t="n">
-        <v>3237.5999</v>
+        <v>9121.110000000001</v>
       </c>
       <c r="N21" t="n">
-        <v>-210.1599</v>
+        <v>-2685.15</v>
       </c>
       <c r="O21" t="n">
-        <v>-6.4912</v>
+        <v>-29.4388</v>
       </c>
       <c r="P21" t="n">
-        <v>1.101</v>
+        <v>2.2313</v>
       </c>
       <c r="Q21" t="n">
-        <v>5.7</v>
+        <v>22.8027</v>
       </c>
       <c r="R21" t="n">
         <v>0</v>
@@ -2478,44 +2482,44 @@
         <v>0</v>
       </c>
       <c r="V21" t="n">
-        <v>5.34</v>
+        <v>15.93</v>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>https://api.etrade.com/v1/accounts/fOTHyxD-9tctDlNfYkhFzA/portfolio/387800975900.json</t>
+          <t>https://api.etrade.com/v1/accounts/fOTHyxD-9tctDlNfYkhFzA/portfolio/415421866900.json</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>https://api.etrade.com/v1/market/quote/BRSP.json</t>
+          <t>https://api.etrade.com/v1/market/quote/MARA.json</t>
         </is>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
-          <t>{'symbol': 'BRSP', 'securityType': 'EQ', 'expiryYear': 0, 'expiryMonth': 0, 'expiryDay': 0, 'strikePrice': 0, 'productId': {'symbol': 'BRSP', 'typeCode': 'EQUITY'}}</t>
+          <t>{'symbol': 'MARA', 'securityType': 'EQ', 'expiryYear': 0, 'expiryMonth': 0, 'expiryDay': 0, 'strikePrice': 0, 'productId': {'symbol': 'MARA', 'typeCode': 'EQUITY'}}</t>
         </is>
       </c>
       <c r="Z21" t="inlineStr">
         <is>
-          <t>{'lastTrade': 5.33, 'lastTradeTime': 1754683800, 'change': -0.01, 'changePct': -0.1872, 'volume': 696953, 'quoteStatus': 'CLOSING'}</t>
+          <t>{'lastTrade': 16.0899, 'lastTradeTime': 1757527585, 'change': 0.1599, 'changePct': 1.0037, 'volume': 42064671, 'quoteStatus': 'REALTIME'}</t>
         </is>
       </c>
       <c r="AA21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>372681778900</v>
+        <v>3154552844</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>BITO</t>
+          <t>MAGS</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>1711080000000</v>
+        <v>1754539200000</v>
       </c>
       <c r="D22" t="n">
-        <v>28.0018</v>
+        <v>58.8051</v>
       </c>
       <c r="E22" t="n">
         <v>0</v>
@@ -2524,7 +2528,7 @@
         <v>0</v>
       </c>
       <c r="G22" t="n">
-        <v>440</v>
+        <v>200</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
@@ -2537,28 +2541,28 @@
         </is>
       </c>
       <c r="J22" t="n">
-        <v>-101.2</v>
+        <v>-18</v>
       </c>
       <c r="K22" t="n">
-        <v>-1.0787</v>
+        <v>-0.1458</v>
       </c>
       <c r="L22" t="n">
-        <v>9279.6</v>
+        <v>12326</v>
       </c>
       <c r="M22" t="n">
-        <v>12320.7999</v>
+        <v>11761.04</v>
       </c>
       <c r="N22" t="n">
-        <v>-3041.1999</v>
+        <v>564.96</v>
       </c>
       <c r="O22" t="n">
-        <v>-24.6834</v>
+        <v>4.8036</v>
       </c>
       <c r="P22" t="n">
-        <v>3.3748</v>
+        <v>4.2734</v>
       </c>
       <c r="Q22" t="n">
-        <v>28.0018</v>
+        <v>58.8052</v>
       </c>
       <c r="R22" t="n">
         <v>0</v>
@@ -2573,44 +2577,44 @@
         <v>0</v>
       </c>
       <c r="V22" t="n">
-        <v>21.32</v>
+        <v>61.72</v>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>https://api.etrade.com/v1/accounts/fOTHyxD-9tctDlNfYkhFzA/portfolio/372681778900.json</t>
+          <t>https://api.etrade.com/v1/accounts/fOTHyxD-9tctDlNfYkhFzA/portfolio/3154552844.json</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>https://api.etrade.com/v1/market/quote/BITO.json</t>
+          <t>https://api.etrade.com/v1/market/quote/MAGS.json</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>{'symbol': 'BITO', 'securityType': 'EQ', 'securitySubType': 'ETF', 'expiryYear': 0, 'expiryMonth': 0, 'expiryDay': 0, 'strikePrice': 0, 'productId': {'symbol': 'BITO', 'typeCode': 'EQUITY'}}</t>
+          <t>{'symbol': 'MAGS', 'securityType': 'EQ', 'securitySubType': 'ETF', 'expiryYear': 0, 'expiryMonth': 0, 'expiryDay': 0, 'strikePrice': 0, 'productId': {'symbol': 'MAGS', 'typeCode': 'EQUITY'}}</t>
         </is>
       </c>
       <c r="Z22" t="inlineStr">
         <is>
-          <t>{'lastTrade': 21.09, 'lastTradeTime': 1754683800, 'change': -0.23, 'changePct': -1.0787, 'volume': 8846203, 'quoteStatus': 'CLOSING'}</t>
+          <t>{'lastTrade': 61.63, 'lastTradeTime': 1757527579, 'change': -0.09, 'changePct': -0.1458, 'volume': 1463379, 'quoteStatus': 'REALTIME'}</t>
         </is>
       </c>
       <c r="AA22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>424714867900</v>
+        <v>387800975900</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>AMZU</t>
+          <t>BRSP</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>1737003600000</v>
+        <v>1719806400000</v>
       </c>
       <c r="D23" t="n">
-        <v>43.8777</v>
+        <v>5.7</v>
       </c>
       <c r="E23" t="n">
         <v>0</v>
@@ -2619,7 +2623,7 @@
         <v>0</v>
       </c>
       <c r="G23" t="n">
-        <v>200</v>
+        <v>568</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
@@ -2632,28 +2636,28 @@
         </is>
       </c>
       <c r="J23" t="n">
-        <v>-32</v>
+        <v>0</v>
       </c>
       <c r="K23" t="n">
-        <v>-0.4318</v>
+        <v>0</v>
       </c>
       <c r="L23" t="n">
-        <v>7378</v>
+        <v>3339.84</v>
       </c>
       <c r="M23" t="n">
-        <v>8775.5499</v>
+        <v>3237.5999</v>
       </c>
       <c r="N23" t="n">
-        <v>-1397.5499</v>
+        <v>102.2399</v>
       </c>
       <c r="O23" t="n">
-        <v>-15.9254</v>
+        <v>3.1578</v>
       </c>
       <c r="P23" t="n">
-        <v>2.6832</v>
+        <v>1.1579</v>
       </c>
       <c r="Q23" t="n">
-        <v>43.8777</v>
+        <v>5.7</v>
       </c>
       <c r="R23" t="n">
         <v>0</v>
@@ -2668,44 +2672,44 @@
         <v>0</v>
       </c>
       <c r="V23" t="n">
-        <v>37.05</v>
+        <v>5.88</v>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>https://api.etrade.com/v1/accounts/fOTHyxD-9tctDlNfYkhFzA/portfolio/424714867900.json</t>
+          <t>https://api.etrade.com/v1/accounts/fOTHyxD-9tctDlNfYkhFzA/portfolio/387800975900.json</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>https://api.etrade.com/v1/market/quote/AMZU.json</t>
+          <t>https://api.etrade.com/v1/market/quote/BRSP.json</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>{'symbol': 'AMZU', 'securityType': 'EQ', 'securitySubType': 'ETF', 'expiryYear': 0, 'expiryMonth': 0, 'expiryDay': 0, 'strikePrice': 0, 'productId': {'symbol': 'AMZU', 'typeCode': 'EQUITY'}}</t>
+          <t>{'symbol': 'BRSP', 'securityType': 'EQ', 'expiryYear': 0, 'expiryMonth': 0, 'expiryDay': 0, 'strikePrice': 0, 'productId': {'symbol': 'BRSP', 'typeCode': 'EQUITY'}}</t>
         </is>
       </c>
       <c r="Z23" t="inlineStr">
         <is>
-          <t>{'lastTrade': 36.89, 'lastTradeTime': 1754684100, 'change': -0.16, 'changePct': -0.4318, 'volume': 1349827, 'quoteStatus': 'CLOSING'}</t>
+          <t>{'lastTrade': 5.88, 'lastTradeTime': 1757527510, 'change': 0, 'changePct': 0, 'volume': 263992, 'quoteStatus': 'REALTIME'}</t>
         </is>
       </c>
       <c r="AA23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>390367652900</v>
+        <v>372681778900</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>AGNC</t>
+          <t>BITO</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>1721102400000</v>
+        <v>1711080000000</v>
       </c>
       <c r="D24" t="n">
-        <v>10.37</v>
+        <v>28.0018</v>
       </c>
       <c r="E24" t="n">
         <v>0</v>
@@ -2714,7 +2718,7 @@
         <v>0</v>
       </c>
       <c r="G24" t="n">
-        <v>736</v>
+        <v>440</v>
       </c>
       <c r="H24" t="inlineStr">
         <is>
@@ -2727,28 +2731,28 @@
         </is>
       </c>
       <c r="J24" t="n">
-        <v>29.44</v>
+        <v>193.5999</v>
       </c>
       <c r="K24" t="n">
-        <v>0.425</v>
+        <v>2.2928</v>
       </c>
       <c r="L24" t="n">
-        <v>6955.1999</v>
+        <v>8637.200000000001</v>
       </c>
       <c r="M24" t="n">
-        <v>7632.3494</v>
+        <v>12320.7999</v>
       </c>
       <c r="N24" t="n">
-        <v>-677.1494</v>
+        <v>-3683.5999</v>
       </c>
       <c r="O24" t="n">
-        <v>-8.872</v>
+        <v>-29.8974</v>
       </c>
       <c r="P24" t="n">
-        <v>2.5295</v>
+        <v>2.9945</v>
       </c>
       <c r="Q24" t="n">
-        <v>10.37</v>
+        <v>28.0018</v>
       </c>
       <c r="R24" t="n">
         <v>0</v>
@@ -2763,53 +2767,53 @@
         <v>0</v>
       </c>
       <c r="V24" t="n">
-        <v>9.41</v>
+        <v>19.19</v>
       </c>
       <c r="W24" t="inlineStr">
         <is>
-          <t>https://api.etrade.com/v1/accounts/fOTHyxD-9tctDlNfYkhFzA/portfolio/390367652900.json</t>
+          <t>https://api.etrade.com/v1/accounts/fOTHyxD-9tctDlNfYkhFzA/portfolio/372681778900.json</t>
         </is>
       </c>
       <c r="X24" t="inlineStr">
         <is>
-          <t>https://api.etrade.com/v1/market/quote/AGNC.json</t>
+          <t>https://api.etrade.com/v1/market/quote/BITO.json</t>
         </is>
       </c>
       <c r="Y24" t="inlineStr">
         <is>
-          <t>{'symbol': 'AGNC', 'securityType': 'EQ', 'expiryYear': 0, 'expiryMonth': 0, 'expiryDay': 0, 'strikePrice': 0, 'productId': {'symbol': 'AGNC', 'typeCode': 'EQUITY'}}</t>
+          <t>{'symbol': 'BITO', 'securityType': 'EQ', 'securitySubType': 'ETF', 'expiryYear': 0, 'expiryMonth': 0, 'expiryDay': 0, 'strikePrice': 0, 'productId': {'symbol': 'BITO', 'typeCode': 'EQUITY'}}</t>
         </is>
       </c>
       <c r="Z24" t="inlineStr">
         <is>
-          <t>{'lastTrade': 9.45, 'lastTradeTime': 1754683200, 'change': 0.04, 'changePct': 0.425, 'volume': 10853057, 'quoteStatus': 'CLOSING'}</t>
+          <t>{'lastTrade': 19.63, 'lastTradeTime': 1757527581, 'change': 0.44, 'changePct': 2.2928, 'volume': 7491527, 'quoteStatus': 'REALTIME'}</t>
         </is>
       </c>
       <c r="AA24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>371438937900</v>
+        <v>9418048844</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>ACP</t>
+          <t>AVL Oct 17 '25 $56 Put</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>1711080000000</v>
+        <v>1757044800000</v>
       </c>
       <c r="D25" t="n">
-        <v>6.6412</v>
+        <v>4.5</v>
       </c>
       <c r="E25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F25" t="n">
-        <v>0</v>
+        <v>0.04</v>
       </c>
       <c r="G25" t="n">
-        <v>1625</v>
+        <v>-2</v>
       </c>
       <c r="H25" t="inlineStr">
         <is>
@@ -2818,32 +2822,32 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>LONG</t>
+          <t>SHORT</t>
         </is>
       </c>
       <c r="J25" t="n">
-        <v>0</v>
+        <v>490</v>
       </c>
       <c r="K25" t="n">
-        <v>0</v>
+        <v>48.0392</v>
       </c>
       <c r="L25" t="n">
-        <v>9668.75</v>
+        <v>-530</v>
       </c>
       <c r="M25" t="n">
-        <v>10791.9987</v>
+        <v>-898.96</v>
       </c>
       <c r="N25" t="n">
-        <v>-1123.2487</v>
+        <v>368.9599</v>
       </c>
       <c r="O25" t="n">
-        <v>-10.4081</v>
+        <v>41.0429</v>
       </c>
       <c r="P25" t="n">
-        <v>3.5164</v>
+        <v>-0.1837</v>
       </c>
       <c r="Q25" t="n">
-        <v>6.6412</v>
+        <v>4.4948</v>
       </c>
       <c r="R25" t="n">
         <v>0</v>
@@ -2858,44 +2862,48 @@
         <v>0</v>
       </c>
       <c r="V25" t="n">
-        <v>5.95</v>
+        <v>5.1</v>
       </c>
       <c r="W25" t="inlineStr">
         <is>
-          <t>https://api.etrade.com/v1/accounts/fOTHyxD-9tctDlNfYkhFzA/portfolio/371438937900.json</t>
+          <t>https://api.etrade.com/v1/accounts/fOTHyxD-9tctDlNfYkhFzA/portfolio/9418048844.json</t>
         </is>
       </c>
       <c r="X25" t="inlineStr">
         <is>
-          <t>https://api.etrade.com/v1/market/quote/ACP.json</t>
+          <t>https://api.etrade.com/v1/market/quote/AVL:2025:10:17:PUT:56.json</t>
         </is>
       </c>
       <c r="Y25" t="inlineStr">
         <is>
-          <t>{'symbol': 'ACP', 'securityType': 'EQ', 'securitySubType': 'CMUT', 'expiryYear': 0, 'expiryMonth': 0, 'expiryDay': 0, 'strikePrice': 0, 'productId': {'symbol': 'ACP', 'typeCode': 'EQUITY'}}</t>
+          <t>{'symbol': 'AVL', 'securityType': 'OPTN', 'callPut': 'PUT', 'expiryYear': 2025, 'expiryMonth': 10, 'expiryDay': 17, 'strikePrice': 56, 'productId': {'symbol': 'AVL', 'typeCode': 'EQUITY'}}</t>
         </is>
       </c>
       <c r="Z25" t="inlineStr">
         <is>
-          <t>{'lastTrade': 5.95, 'lastTradeTime': 1754683800, 'change': 0, 'changePct': 0, 'volume': 330657, 'quoteStatus': 'CLOSING'}</t>
-        </is>
-      </c>
-      <c r="AA25" t="inlineStr"/>
+          <t>{'lastTrade': 5.1, 'lastTradeTime': 1757527581, 'change': -2.45, 'changePct': -48.0392, 'volume': 0, 'quoteStatus': 'REALTIME'}</t>
+        </is>
+      </c>
+      <c r="AA25" t="inlineStr">
+        <is>
+          <t>AVL---251017P00056000</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>444464528900</v>
+        <v>6073887844</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>DOCS Aug 15 '25 $45 Put</t>
+          <t>AMZU Oct 17 '25 $36 Put</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>1744776000000</v>
+        <v>1755662400000</v>
       </c>
       <c r="D26" t="n">
-        <v>5.45</v>
+        <v>2.5</v>
       </c>
       <c r="E26" t="n">
         <v>0.5</v>
@@ -2904,7 +2912,7 @@
         <v>0.02</v>
       </c>
       <c r="G26" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="H26" t="inlineStr">
         <is>
@@ -2913,32 +2921,32 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>LONG</t>
+          <t>SHORT</t>
         </is>
       </c>
       <c r="J26" t="n">
-        <v>-2.5</v>
+        <v>-57.5</v>
       </c>
       <c r="K26" t="n">
-        <v>-25</v>
+        <v>-69.6969</v>
       </c>
       <c r="L26" t="n">
-        <v>7.5</v>
+        <v>-140</v>
       </c>
       <c r="M26" t="n">
-        <v>545.5199</v>
+        <v>-249.4799</v>
       </c>
       <c r="N26" t="n">
-        <v>-538.0199</v>
+        <v>109.48</v>
       </c>
       <c r="O26" t="n">
-        <v>-98.6251</v>
+        <v>43.8832</v>
       </c>
       <c r="P26" t="n">
-        <v>0.0027</v>
+        <v>-0.0485</v>
       </c>
       <c r="Q26" t="n">
-        <v>5.4552</v>
+        <v>2.4948</v>
       </c>
       <c r="R26" t="n">
         <v>0</v>
@@ -2953,48 +2961,48 @@
         <v>0</v>
       </c>
       <c r="V26" t="n">
-        <v>0.1</v>
+        <v>0.825</v>
       </c>
       <c r="W26" t="inlineStr">
         <is>
-          <t>https://api.etrade.com/v1/accounts/fOTHyxD-9tctDlNfYkhFzA/portfolio/444464528900.json</t>
+          <t>https://api.etrade.com/v1/accounts/fOTHyxD-9tctDlNfYkhFzA/portfolio/6073887844.json</t>
         </is>
       </c>
       <c r="X26" t="inlineStr">
         <is>
-          <t>https://api.etrade.com/v1/market/quote/DOCS:2025:8:15:PUT:45.json</t>
+          <t>https://api.etrade.com/v1/market/quote/AMZU:2025:10:17:PUT:36.json</t>
         </is>
       </c>
       <c r="Y26" t="inlineStr">
         <is>
-          <t>{'symbol': 'DOCS', 'securityType': 'OPTN', 'callPut': 'PUT', 'expiryYear': 2025, 'expiryMonth': 8, 'expiryDay': 15, 'strikePrice': 45, 'productId': {'symbol': 'DOCS', 'typeCode': 'EQUITY'}}</t>
+          <t>{'symbol': 'AMZU', 'securityType': 'OPTN', 'callPut': 'PUT', 'expiryYear': 2025, 'expiryMonth': 10, 'expiryDay': 17, 'strikePrice': 36, 'productId': {'symbol': 'AMZU', 'typeCode': 'EQUITY'}}</t>
         </is>
       </c>
       <c r="Z26" t="inlineStr">
         <is>
-          <t>{'lastTrade': 0.08, 'lastTradeTime': 1754683195, 'change': -0.025, 'changePct': -25, 'volume': 66, 'quoteStatus': 'REALTIME'}</t>
+          <t>{'lastTrade': 1.35, 'lastTradeTime': 1757527585, 'change': 0.575, 'changePct': 69.6969, 'volume': 176, 'quoteStatus': 'REALTIME'}</t>
         </is>
       </c>
       <c r="AA26" t="inlineStr">
         <is>
-          <t>DOCS--250815P00045000</t>
+          <t>AMZU--251017P00036000</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>383722115900</v>
+        <v>424714867900</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>DSL</t>
+          <t>AMZU</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>1717646400000</v>
+        <v>1737003600000</v>
       </c>
       <c r="D27" t="n">
-        <v>12.5</v>
+        <v>43.8777</v>
       </c>
       <c r="E27" t="n">
         <v>0</v>
@@ -3003,7 +3011,7 @@
         <v>0</v>
       </c>
       <c r="G27" t="n">
-        <v>260</v>
+        <v>200</v>
       </c>
       <c r="H27" t="inlineStr">
         <is>
@@ -3016,28 +3024,28 @@
         </is>
       </c>
       <c r="J27" t="n">
-        <v>28.6</v>
+        <v>-520</v>
       </c>
       <c r="K27" t="n">
-        <v>0.9023</v>
+        <v>-6.2484</v>
       </c>
       <c r="L27" t="n">
-        <v>3198</v>
+        <v>7802</v>
       </c>
       <c r="M27" t="n">
-        <v>3250</v>
+        <v>8775.5499</v>
       </c>
       <c r="N27" t="n">
-        <v>-52</v>
+        <v>-973.5499</v>
       </c>
       <c r="O27" t="n">
-        <v>-1.6</v>
+        <v>-11.0938</v>
       </c>
       <c r="P27" t="n">
-        <v>1.163</v>
+        <v>2.7049</v>
       </c>
       <c r="Q27" t="n">
-        <v>12.5</v>
+        <v>43.8777</v>
       </c>
       <c r="R27" t="n">
         <v>0</v>
@@ -3052,44 +3060,44 @@
         <v>0</v>
       </c>
       <c r="V27" t="n">
-        <v>12.19</v>
+        <v>41.61</v>
       </c>
       <c r="W27" t="inlineStr">
         <is>
-          <t>https://api.etrade.com/v1/accounts/fOTHyxD-9tctDlNfYkhFzA/portfolio/383722115900.json</t>
+          <t>https://api.etrade.com/v1/accounts/fOTHyxD-9tctDlNfYkhFzA/portfolio/424714867900.json</t>
         </is>
       </c>
       <c r="X27" t="inlineStr">
         <is>
-          <t>https://api.etrade.com/v1/market/quote/DSL.json</t>
+          <t>https://api.etrade.com/v1/market/quote/AMZU.json</t>
         </is>
       </c>
       <c r="Y27" t="inlineStr">
         <is>
-          <t>{'symbol': 'DSL', 'securityType': 'EQ', 'securitySubType': 'CMUT', 'expiryYear': 0, 'expiryMonth': 0, 'expiryDay': 0, 'strikePrice': 0, 'productId': {'symbol': 'DSL', 'typeCode': 'EQUITY'}}</t>
+          <t>{'symbol': 'AMZU', 'securityType': 'EQ', 'securitySubType': 'ETF', 'expiryYear': 0, 'expiryMonth': 0, 'expiryDay': 0, 'strikePrice': 0, 'productId': {'symbol': 'AMZU', 'typeCode': 'EQUITY'}}</t>
         </is>
       </c>
       <c r="Z27" t="inlineStr">
         <is>
-          <t>{'lastTrade': 12.3, 'lastTradeTime': 1754683800, 'change': 0.11, 'changePct': 0.9023, 'volume': 314851, 'quoteStatus': 'CLOSING'}</t>
+          <t>{'lastTrade': 39.01, 'lastTradeTime': 1757527580, 'change': -2.6, 'changePct': -6.2484, 'volume': 2514013, 'quoteStatus': 'REALTIME'}</t>
         </is>
       </c>
       <c r="AA27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>3154552844</v>
+        <v>390367652900</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>MAGS</t>
+          <t>AGNC</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>1754625600000</v>
+        <v>1721102400000</v>
       </c>
       <c r="D28" t="n">
-        <v>58.8051</v>
+        <v>10.37</v>
       </c>
       <c r="E28" t="n">
         <v>0</v>
@@ -3098,7 +3106,7 @@
         <v>0</v>
       </c>
       <c r="G28" t="n">
-        <v>200</v>
+        <v>736</v>
       </c>
       <c r="H28" t="inlineStr">
         <is>
@@ -3111,28 +3119,28 @@
         </is>
       </c>
       <c r="J28" t="n">
-        <v>194</v>
+        <v>-11.0399</v>
       </c>
       <c r="K28" t="n">
-        <v>1.6451</v>
+        <v>-0.1449</v>
       </c>
       <c r="L28" t="n">
-        <v>11986</v>
+        <v>7606.56</v>
       </c>
       <c r="M28" t="n">
-        <v>11761.04</v>
+        <v>7632.3494</v>
       </c>
       <c r="N28" t="n">
-        <v>224.96</v>
+        <v>-25.7894</v>
       </c>
       <c r="O28" t="n">
-        <v>1.9127</v>
+        <v>-0.3378</v>
       </c>
       <c r="P28" t="n">
-        <v>4.3591</v>
+        <v>2.6372</v>
       </c>
       <c r="Q28" t="n">
-        <v>58.8052</v>
+        <v>10.37</v>
       </c>
       <c r="R28" t="n">
         <v>0</v>
@@ -3147,53 +3155,53 @@
         <v>0</v>
       </c>
       <c r="V28" t="n">
-        <v>58.96</v>
+        <v>10.35</v>
       </c>
       <c r="W28" t="inlineStr">
         <is>
-          <t>https://api.etrade.com/v1/accounts/fOTHyxD-9tctDlNfYkhFzA/portfolio/3154552844.json</t>
+          <t>https://api.etrade.com/v1/accounts/fOTHyxD-9tctDlNfYkhFzA/portfolio/390367652900.json</t>
         </is>
       </c>
       <c r="X28" t="inlineStr">
         <is>
-          <t>https://api.etrade.com/v1/market/quote/MAGS.json</t>
+          <t>https://api.etrade.com/v1/market/quote/AGNC.json</t>
         </is>
       </c>
       <c r="Y28" t="inlineStr">
         <is>
-          <t>{'symbol': 'MAGS', 'securityType': 'EQ', 'securitySubType': 'ETF', 'expiryYear': 0, 'expiryMonth': 0, 'expiryDay': 0, 'strikePrice': 0, 'productId': {'symbol': 'MAGS', 'typeCode': 'EQUITY'}}</t>
+          <t>{'symbol': 'AGNC', 'securityType': 'EQ', 'expiryYear': 0, 'expiryMonth': 0, 'expiryDay': 0, 'strikePrice': 0, 'productId': {'symbol': 'AGNC', 'typeCode': 'EQUITY'}}</t>
         </is>
       </c>
       <c r="Z28" t="inlineStr">
         <is>
-          <t>{'lastTrade': 59.93, 'lastTradeTime': 1754683804, 'change': 0.97, 'changePct': 1.6451, 'volume': 3590580, 'quoteStatus': 'CLOSING'}</t>
+          <t>{'lastTrade': 10.335, 'lastTradeTime': 1757527576, 'change': -0.015, 'changePct': -0.1449, 'volume': 13566152, 'quoteStatus': 'REALTIME'}</t>
         </is>
       </c>
       <c r="AA28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>465022079900</v>
+        <v>371438937900</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>EQT Sep 19 '25 $60 Put</t>
+          <t>ACP</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>1753243200000</v>
+        <v>1711080000000</v>
       </c>
       <c r="D29" t="n">
-        <v>8.6999</v>
+        <v>6.6412</v>
       </c>
       <c r="E29" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="F29" t="n">
-        <v>0.02</v>
+        <v>0</v>
       </c>
       <c r="G29" t="n">
-        <v>-1</v>
+        <v>1625</v>
       </c>
       <c r="H29" t="inlineStr">
         <is>
@@ -3202,32 +3210,32 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>SHORT</t>
+          <t>LONG</t>
         </is>
       </c>
       <c r="J29" t="n">
-        <v>0</v>
+        <v>-9.9124</v>
       </c>
       <c r="K29" t="n">
-        <v>0</v>
+        <v>-0.1033</v>
       </c>
       <c r="L29" t="n">
-        <v>-877.5</v>
+        <v>9577.5874</v>
       </c>
       <c r="M29" t="n">
-        <v>-869.48</v>
+        <v>10791.9987</v>
       </c>
       <c r="N29" t="n">
-        <v>-8.0199</v>
+        <v>-1214.4112</v>
       </c>
       <c r="O29" t="n">
-        <v>-0.9223</v>
+        <v>-11.2528</v>
       </c>
       <c r="P29" t="n">
-        <v>-0.3191</v>
+        <v>3.3206</v>
       </c>
       <c r="Q29" t="n">
-        <v>8.694800000000001</v>
+        <v>6.6412</v>
       </c>
       <c r="R29" t="n">
         <v>0</v>
@@ -3242,48 +3250,44 @@
         <v>0</v>
       </c>
       <c r="V29" t="n">
-        <v>8.775</v>
+        <v>5.9</v>
       </c>
       <c r="W29" t="inlineStr">
         <is>
-          <t>https://api.etrade.com/v1/accounts/fOTHyxD-9tctDlNfYkhFzA/portfolio/465022079900.json</t>
+          <t>https://api.etrade.com/v1/accounts/fOTHyxD-9tctDlNfYkhFzA/portfolio/371438937900.json</t>
         </is>
       </c>
       <c r="X29" t="inlineStr">
         <is>
-          <t>https://api.etrade.com/v1/market/quote/EQT:2025:9:19:PUT:60.json</t>
+          <t>https://api.etrade.com/v1/market/quote/ACP.json</t>
         </is>
       </c>
       <c r="Y29" t="inlineStr">
         <is>
-          <t>{'symbol': 'EQT', 'securityType': 'OPTN', 'callPut': 'PUT', 'expiryYear': 2025, 'expiryMonth': 9, 'expiryDay': 19, 'strikePrice': 60, 'productId': {'symbol': 'EQT', 'typeCode': 'EQUITY'}}</t>
+          <t>{'symbol': 'ACP', 'securityType': 'EQ', 'securitySubType': 'CMUT', 'expiryYear': 0, 'expiryMonth': 0, 'expiryDay': 0, 'strikePrice': 0, 'productId': {'symbol': 'ACP', 'typeCode': 'EQUITY'}}</t>
         </is>
       </c>
       <c r="Z29" t="inlineStr">
         <is>
-          <t>{'lastTrade': 9.0, 'lastTradeTime': 1754683199, 'change': 0, 'changePct': 0, 'volume': 3, 'quoteStatus': 'REALTIME'}</t>
-        </is>
-      </c>
-      <c r="AA29" t="inlineStr">
-        <is>
-          <t>EQT---250919P00060000</t>
-        </is>
-      </c>
+          <t>{'lastTrade': 5.8939, 'lastTradeTime': 1757527583, 'change': -0.0061, 'changePct': -0.1033, 'volume': 350706, 'quoteStatus': 'REALTIME'}</t>
+        </is>
+      </c>
+      <c r="AA29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>455519818900</v>
+        <v>374009142900</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>EQT</t>
+          <t>CHMI</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>1749528000000</v>
+        <v>1712635200000</v>
       </c>
       <c r="D30" t="n">
-        <v>55.4052</v>
+        <v>3.3992</v>
       </c>
       <c r="E30" t="n">
         <v>0</v>
@@ -3292,7 +3296,7 @@
         <v>0</v>
       </c>
       <c r="G30" t="n">
-        <v>100</v>
+        <v>2425</v>
       </c>
       <c r="H30" t="inlineStr">
         <is>
@@ -3305,28 +3309,28 @@
         </is>
       </c>
       <c r="J30" t="n">
-        <v>5</v>
+        <v>133.375</v>
       </c>
       <c r="K30" t="n">
-        <v>0.0975</v>
+        <v>1.8835</v>
       </c>
       <c r="L30" t="n">
-        <v>5129</v>
+        <v>7214.375</v>
       </c>
       <c r="M30" t="n">
-        <v>5540.52</v>
+        <v>8243.249100000001</v>
       </c>
       <c r="N30" t="n">
-        <v>-411.5199</v>
+        <v>-1028.8741</v>
       </c>
       <c r="O30" t="n">
-        <v>-7.4274</v>
+        <v>-12.4814</v>
       </c>
       <c r="P30" t="n">
-        <v>1.8653</v>
+        <v>2.5012</v>
       </c>
       <c r="Q30" t="n">
-        <v>55.4052</v>
+        <v>3.3992</v>
       </c>
       <c r="R30" t="n">
         <v>0</v>
@@ -3341,44 +3345,44 @@
         <v>0</v>
       </c>
       <c r="V30" t="n">
-        <v>51.24</v>
+        <v>2.92</v>
       </c>
       <c r="W30" t="inlineStr">
         <is>
-          <t>https://api.etrade.com/v1/accounts/fOTHyxD-9tctDlNfYkhFzA/portfolio/455519818900.json</t>
+          <t>https://api.etrade.com/v1/accounts/fOTHyxD-9tctDlNfYkhFzA/portfolio/374009142900.json</t>
         </is>
       </c>
       <c r="X30" t="inlineStr">
         <is>
-          <t>https://api.etrade.com/v1/market/quote/EQT.json</t>
+          <t>https://api.etrade.com/v1/market/quote/CHMI.json</t>
         </is>
       </c>
       <c r="Y30" t="inlineStr">
         <is>
-          <t>{'symbol': 'EQT', 'securityType': 'EQ', 'expiryYear': 0, 'expiryMonth': 0, 'expiryDay': 0, 'strikePrice': 0, 'productId': {'symbol': 'EQT', 'typeCode': 'EQUITY'}}</t>
+          <t>{'symbol': 'CHMI', 'securityType': 'EQ', 'expiryYear': 0, 'expiryMonth': 0, 'expiryDay': 0, 'strikePrice': 0, 'productId': {'symbol': 'CHMI', 'typeCode': 'EQUITY'}}</t>
         </is>
       </c>
       <c r="Z30" t="inlineStr">
         <is>
-          <t>{'lastTrade': 51.29, 'lastTradeTime': 1754683800, 'change': 0.05, 'changePct': 0.0975, 'volume': 4540308, 'quoteStatus': 'CLOSING'}</t>
+          <t>{'lastTrade': 2.975, 'lastTradeTime': 1757527553, 'change': 0.055, 'changePct': 1.8835, 'volume': 125066, 'quoteStatus': 'REALTIME'}</t>
         </is>
       </c>
       <c r="AA30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>384696870900</v>
+        <v>383722115900</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>EIC</t>
+          <t>DSL</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>1718164800000</v>
+        <v>1717646400000</v>
       </c>
       <c r="D31" t="n">
-        <v>15.65</v>
+        <v>12.5</v>
       </c>
       <c r="E31" t="n">
         <v>0</v>
@@ -3387,7 +3391,7 @@
         <v>0</v>
       </c>
       <c r="G31" t="n">
-        <v>466</v>
+        <v>260</v>
       </c>
       <c r="H31" t="inlineStr">
         <is>
@@ -3400,28 +3404,28 @@
         </is>
       </c>
       <c r="J31" t="n">
-        <v>-32.6199</v>
+        <v>-9.0999</v>
       </c>
       <c r="K31" t="n">
-        <v>-0.5714</v>
+        <v>-0.2777</v>
       </c>
       <c r="L31" t="n">
-        <v>5675.88</v>
+        <v>3266.9</v>
       </c>
       <c r="M31" t="n">
-        <v>7292.8999</v>
+        <v>3250</v>
       </c>
       <c r="N31" t="n">
-        <v>-1617.0199</v>
+        <v>16.8999</v>
       </c>
       <c r="O31" t="n">
-        <v>-22.1725</v>
+        <v>0.52</v>
       </c>
       <c r="P31" t="n">
-        <v>2.0642</v>
+        <v>1.1326</v>
       </c>
       <c r="Q31" t="n">
-        <v>15.65</v>
+        <v>12.5</v>
       </c>
       <c r="R31" t="n">
         <v>0</v>
@@ -3436,44 +3440,44 @@
         <v>0</v>
       </c>
       <c r="V31" t="n">
-        <v>12.25</v>
+        <v>12.6</v>
       </c>
       <c r="W31" t="inlineStr">
         <is>
-          <t>https://api.etrade.com/v1/accounts/fOTHyxD-9tctDlNfYkhFzA/portfolio/384696870900.json</t>
+          <t>https://api.etrade.com/v1/accounts/fOTHyxD-9tctDlNfYkhFzA/portfolio/383722115900.json</t>
         </is>
       </c>
       <c r="X31" t="inlineStr">
         <is>
-          <t>https://api.etrade.com/v1/market/quote/EIC.json</t>
+          <t>https://api.etrade.com/v1/market/quote/DSL.json</t>
         </is>
       </c>
       <c r="Y31" t="inlineStr">
         <is>
-          <t>{'symbol': 'EIC', 'securityType': 'EQ', 'securitySubType': 'CMUT', 'expiryYear': 0, 'expiryMonth': 0, 'expiryDay': 0, 'strikePrice': 0, 'productId': {'symbol': 'EIC', 'typeCode': 'EQUITY'}}</t>
+          <t>{'symbol': 'DSL', 'securityType': 'EQ', 'securitySubType': 'CMUT', 'expiryYear': 0, 'expiryMonth': 0, 'expiryDay': 0, 'strikePrice': 0, 'productId': {'symbol': 'DSL', 'typeCode': 'EQUITY'}}</t>
         </is>
       </c>
       <c r="Z31" t="inlineStr">
         <is>
-          <t>{'lastTrade': 12.18, 'lastTradeTime': 1754683800, 'change': -0.07, 'changePct': -0.5714, 'volume': 502826, 'quoteStatus': 'CLOSING'}</t>
+          <t>{'lastTrade': 12.565, 'lastTradeTime': 1757527585, 'change': -0.035, 'changePct': -0.2777, 'volume': 212155, 'quoteStatus': 'REALTIME'}</t>
         </is>
       </c>
       <c r="AA31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>384160526900</v>
+        <v>376120873900</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>ECC</t>
+          <t>DX</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>1717992000000</v>
+        <v>1713844800000</v>
       </c>
       <c r="D32" t="n">
-        <v>9.813800000000001</v>
+        <v>11.9142</v>
       </c>
       <c r="E32" t="n">
         <v>0</v>
@@ -3482,7 +3486,7 @@
         <v>0</v>
       </c>
       <c r="G32" t="n">
-        <v>1142</v>
+        <v>625</v>
       </c>
       <c r="H32" t="inlineStr">
         <is>
@@ -3495,28 +3499,28 @@
         </is>
       </c>
       <c r="J32" t="n">
-        <v>-205.56</v>
+        <v>-90.625</v>
       </c>
       <c r="K32" t="n">
-        <v>-2.8081</v>
+        <v>-1.124</v>
       </c>
       <c r="L32" t="n">
-        <v>7114.6599</v>
+        <v>7971.875</v>
       </c>
       <c r="M32" t="n">
-        <v>11207.3698</v>
+        <v>7446.3893</v>
       </c>
       <c r="N32" t="n">
-        <v>-4092.7098</v>
+        <v>525.4856</v>
       </c>
       <c r="O32" t="n">
-        <v>-36.518</v>
+        <v>7.0569</v>
       </c>
       <c r="P32" t="n">
-        <v>2.5875</v>
+        <v>2.7638</v>
       </c>
       <c r="Q32" t="n">
-        <v>9.813800000000001</v>
+        <v>11.9142</v>
       </c>
       <c r="R32" t="n">
         <v>0</v>
@@ -3531,53 +3535,53 @@
         <v>0</v>
       </c>
       <c r="V32" t="n">
-        <v>6.41</v>
+        <v>12.9</v>
       </c>
       <c r="W32" t="inlineStr">
         <is>
-          <t>https://api.etrade.com/v1/accounts/fOTHyxD-9tctDlNfYkhFzA/portfolio/384160526900.json</t>
+          <t>https://api.etrade.com/v1/accounts/fOTHyxD-9tctDlNfYkhFzA/portfolio/376120873900.json</t>
         </is>
       </c>
       <c r="X32" t="inlineStr">
         <is>
-          <t>https://api.etrade.com/v1/market/quote/ECC.json</t>
+          <t>https://api.etrade.com/v1/market/quote/DX.json</t>
         </is>
       </c>
       <c r="Y32" t="inlineStr">
         <is>
-          <t>{'symbol': 'ECC', 'securityType': 'EQ', 'securitySubType': 'CMUT', 'expiryYear': 0, 'expiryMonth': 0, 'expiryDay': 0, 'strikePrice': 0, 'productId': {'symbol': 'ECC', 'typeCode': 'EQUITY'}}</t>
+          <t>{'symbol': 'DX', 'securityType': 'EQ', 'expiryYear': 0, 'expiryMonth': 0, 'expiryDay': 0, 'strikePrice': 0, 'productId': {'symbol': 'DX', 'typeCode': 'EQUITY'}}</t>
         </is>
       </c>
       <c r="Z32" t="inlineStr">
         <is>
-          <t>{'lastTrade': 6.23, 'lastTradeTime': 1754683800, 'change': -0.18, 'changePct': -2.8081, 'volume': 6605946, 'quoteStatus': 'CLOSING'}</t>
+          <t>{'lastTrade': 12.755, 'lastTradeTime': 1757527552, 'change': -0.145, 'changePct': -1.124, 'volume': 1955832, 'quoteStatus': 'REALTIME'}</t>
         </is>
       </c>
       <c r="AA32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>376120873900</v>
+        <v>6163695844</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>DX</t>
+          <t>IBKR Oct 17 '25 $70 Put</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>1713844800000</v>
+        <v>1755662400000</v>
       </c>
       <c r="D33" t="n">
-        <v>11.9142</v>
+        <v>9</v>
       </c>
       <c r="E33" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="F33" t="n">
-        <v>0</v>
+        <v>0.02</v>
       </c>
       <c r="G33" t="n">
-        <v>625</v>
+        <v>-1</v>
       </c>
       <c r="H33" t="inlineStr">
         <is>
@@ -3586,32 +3590,32 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>LONG</t>
+          <t>SHORT</t>
         </is>
       </c>
       <c r="J33" t="n">
-        <v>56.25</v>
+        <v>40</v>
       </c>
       <c r="K33" t="n">
-        <v>0.7299</v>
+        <v>4.878</v>
       </c>
       <c r="L33" t="n">
-        <v>7762.5</v>
+        <v>-780</v>
       </c>
       <c r="M33" t="n">
-        <v>7446.3893</v>
+        <v>-899.48</v>
       </c>
       <c r="N33" t="n">
-        <v>316.1106</v>
+        <v>119.48</v>
       </c>
       <c r="O33" t="n">
-        <v>4.2451</v>
+        <v>13.2832</v>
       </c>
       <c r="P33" t="n">
-        <v>2.8231</v>
+        <v>-0.2704</v>
       </c>
       <c r="Q33" t="n">
-        <v>11.9142</v>
+        <v>8.9948</v>
       </c>
       <c r="R33" t="n">
         <v>0</v>
@@ -3626,44 +3630,48 @@
         <v>0</v>
       </c>
       <c r="V33" t="n">
-        <v>12.33</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="W33" t="inlineStr">
         <is>
-          <t>https://api.etrade.com/v1/accounts/fOTHyxD-9tctDlNfYkhFzA/portfolio/376120873900.json</t>
+          <t>https://api.etrade.com/v1/accounts/fOTHyxD-9tctDlNfYkhFzA/portfolio/6163695844.json</t>
         </is>
       </c>
       <c r="X33" t="inlineStr">
         <is>
-          <t>https://api.etrade.com/v1/market/quote/DX.json</t>
+          <t>https://api.etrade.com/v1/market/quote/IBKR:2025:10:17:PUT:70.json</t>
         </is>
       </c>
       <c r="Y33" t="inlineStr">
         <is>
-          <t>{'symbol': 'DX', 'securityType': 'EQ', 'expiryYear': 0, 'expiryMonth': 0, 'expiryDay': 0, 'strikePrice': 0, 'productId': {'symbol': 'DX', 'typeCode': 'EQUITY'}}</t>
+          <t>{'symbol': 'IBKR', 'securityType': 'OPTN', 'callPut': 'PUT', 'expiryYear': 2025, 'expiryMonth': 10, 'expiryDay': 17, 'strikePrice': 70, 'productId': {'symbol': 'IBKR', 'typeCode': 'EQUITY'}}</t>
         </is>
       </c>
       <c r="Z33" t="inlineStr">
         <is>
-          <t>{'lastTrade': 12.42, 'lastTradeTime': 1754683800, 'change': 0.09, 'changePct': 0.7299, 'volume': 2549287, 'quoteStatus': 'CLOSING'}</t>
-        </is>
-      </c>
-      <c r="AA33" t="inlineStr"/>
+          <t>{'lastTrade': 8.2, 'lastTradeTime': 1757527585, 'change': -0.4, 'changePct': -4.878, 'volume': 0, 'quoteStatus': 'REALTIME'}</t>
+        </is>
+      </c>
+      <c r="AA33" t="inlineStr">
+        <is>
+          <t>IBKR--251017P00070000</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>385208533900</v>
+        <v>9504861844</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>SVOL</t>
+          <t>IBKR</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>1718337600000</v>
+        <v>1757044800000</v>
       </c>
       <c r="D34" t="n">
-        <v>22.3287</v>
+        <v>60.7</v>
       </c>
       <c r="E34" t="n">
         <v>0</v>
@@ -3672,7 +3680,7 @@
         <v>0</v>
       </c>
       <c r="G34" t="n">
-        <v>552</v>
+        <v>100</v>
       </c>
       <c r="H34" t="inlineStr">
         <is>
@@ -3685,28 +3693,28 @@
         </is>
       </c>
       <c r="J34" t="n">
-        <v>88.3199</v>
+        <v>46</v>
       </c>
       <c r="K34" t="n">
-        <v>0.9484</v>
+        <v>0.7393999999999999</v>
       </c>
       <c r="L34" t="n">
-        <v>9400.5599</v>
+        <v>6267</v>
       </c>
       <c r="M34" t="n">
-        <v>12325.4898</v>
+        <v>6070</v>
       </c>
       <c r="N34" t="n">
-        <v>-2924.9298</v>
+        <v>197</v>
       </c>
       <c r="O34" t="n">
-        <v>-23.7307</v>
+        <v>3.2454</v>
       </c>
       <c r="P34" t="n">
-        <v>3.4188</v>
+        <v>2.1728</v>
       </c>
       <c r="Q34" t="n">
-        <v>22.3287</v>
+        <v>60.7</v>
       </c>
       <c r="R34" t="n">
         <v>0</v>
@@ -3721,29 +3729,607 @@
         <v>0</v>
       </c>
       <c r="V34" t="n">
-        <v>16.87</v>
+        <v>62.21</v>
       </c>
       <c r="W34" t="inlineStr">
         <is>
-          <t>https://api.etrade.com/v1/accounts/fOTHyxD-9tctDlNfYkhFzA/portfolio/385208533900.json</t>
+          <t>https://api.etrade.com/v1/accounts/fOTHyxD-9tctDlNfYkhFzA/portfolio/9504861844.json</t>
         </is>
       </c>
       <c r="X34" t="inlineStr">
         <is>
-          <t>https://api.etrade.com/v1/market/quote/SVOL.json</t>
+          <t>https://api.etrade.com/v1/market/quote/IBKR.json</t>
         </is>
       </c>
       <c r="Y34" t="inlineStr">
         <is>
-          <t>{'symbol': 'SVOL', 'securityType': 'EQ', 'securitySubType': 'ETF', 'expiryYear': 0, 'expiryMonth': 0, 'expiryDay': 0, 'strikePrice': 0, 'productId': {'symbol': 'SVOL', 'typeCode': 'EQUITY'}}</t>
+          <t>{'symbol': 'IBKR', 'securityType': 'EQ', 'expiryYear': 0, 'expiryMonth': 0, 'expiryDay': 0, 'strikePrice': 0, 'productId': {'symbol': 'IBKR', 'typeCode': 'EQUITY'}}</t>
         </is>
       </c>
       <c r="Z34" t="inlineStr">
         <is>
-          <t>{'lastTrade': 17.03, 'lastTradeTime': 1754683800, 'change': 0.16, 'changePct': 0.9484, 'volume': 549113, 'quoteStatus': 'CLOSING'}</t>
+          <t>{'lastTrade': 62.67, 'lastTradeTime': 1757527583, 'change': 0.46, 'changePct': 0.7394, 'volume': 2339561, 'quoteStatus': 'REALTIME'}</t>
         </is>
       </c>
       <c r="AA34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>9052804844</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>HSAI Oct 17 '25 $35 Put</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>1756872000000</v>
+      </c>
+      <c r="D35" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="E35" t="n">
+        <v>1</v>
+      </c>
+      <c r="F35" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="G35" t="n">
+        <v>-2</v>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>TYPE2</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="J35" t="n">
+        <v>-100</v>
+      </c>
+      <c r="K35" t="n">
+        <v>-6.8965</v>
+      </c>
+      <c r="L35" t="n">
+        <v>-1550</v>
+      </c>
+      <c r="M35" t="n">
+        <v>-1898.96</v>
+      </c>
+      <c r="N35" t="n">
+        <v>348.9599</v>
+      </c>
+      <c r="O35" t="n">
+        <v>18.3763</v>
+      </c>
+      <c r="P35" t="n">
+        <v>-0.5373</v>
+      </c>
+      <c r="Q35" t="n">
+        <v>9.4948</v>
+      </c>
+      <c r="R35" t="n">
+        <v>0</v>
+      </c>
+      <c r="S35" t="n">
+        <v>0</v>
+      </c>
+      <c r="T35" t="n">
+        <v>0</v>
+      </c>
+      <c r="U35" t="n">
+        <v>0</v>
+      </c>
+      <c r="V35" t="n">
+        <v>7.25</v>
+      </c>
+      <c r="W35" t="inlineStr">
+        <is>
+          <t>https://api.etrade.com/v1/accounts/fOTHyxD-9tctDlNfYkhFzA/portfolio/9052804844.json</t>
+        </is>
+      </c>
+      <c r="X35" t="inlineStr">
+        <is>
+          <t>https://api.etrade.com/v1/market/quote/HSAI:2025:10:17:PUT:35.json</t>
+        </is>
+      </c>
+      <c r="Y35" t="inlineStr">
+        <is>
+          <t>{'symbol': 'HSAI', 'securityType': 'OPTN', 'callPut': 'PUT', 'expiryYear': 2025, 'expiryMonth': 10, 'expiryDay': 17, 'strikePrice': 35, 'productId': {'symbol': 'HSAI', 'typeCode': 'EQUITY'}}</t>
+        </is>
+      </c>
+      <c r="Z35" t="inlineStr">
+        <is>
+          <t>{'lastTrade': 7.25, 'lastTradeTime': 1757527576, 'change': 0.5, 'changePct': 6.8965, 'volume': 0, 'quoteStatus': 'REALTIME'}</t>
+        </is>
+      </c>
+      <c r="AA35" t="inlineStr">
+        <is>
+          <t>HSAI--251017P00035000</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>8867139844</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>HSAI</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>1756872000000</v>
+      </c>
+      <c r="D36" t="n">
+        <v>26.26</v>
+      </c>
+      <c r="E36" t="n">
+        <v>0</v>
+      </c>
+      <c r="F36" t="n">
+        <v>0</v>
+      </c>
+      <c r="G36" t="n">
+        <v>200</v>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>TYPE2</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="J36" t="n">
+        <v>-145.24</v>
+      </c>
+      <c r="K36" t="n">
+        <v>-2.5224</v>
+      </c>
+      <c r="L36" t="n">
+        <v>5612.76</v>
+      </c>
+      <c r="M36" t="n">
+        <v>5252</v>
+      </c>
+      <c r="N36" t="n">
+        <v>360.7599</v>
+      </c>
+      <c r="O36" t="n">
+        <v>6.869</v>
+      </c>
+      <c r="P36" t="n">
+        <v>1.9459</v>
+      </c>
+      <c r="Q36" t="n">
+        <v>26.26</v>
+      </c>
+      <c r="R36" t="n">
+        <v>0</v>
+      </c>
+      <c r="S36" t="n">
+        <v>0</v>
+      </c>
+      <c r="T36" t="n">
+        <v>0</v>
+      </c>
+      <c r="U36" t="n">
+        <v>0</v>
+      </c>
+      <c r="V36" t="n">
+        <v>28.79</v>
+      </c>
+      <c r="W36" t="inlineStr">
+        <is>
+          <t>https://api.etrade.com/v1/accounts/fOTHyxD-9tctDlNfYkhFzA/portfolio/8867139844.json</t>
+        </is>
+      </c>
+      <c r="X36" t="inlineStr">
+        <is>
+          <t>https://api.etrade.com/v1/market/quote/HSAI.json</t>
+        </is>
+      </c>
+      <c r="Y36" t="inlineStr">
+        <is>
+          <t>{'symbol': 'HSAI', 'securityType': 'EQ', 'expiryYear': 0, 'expiryMonth': 0, 'expiryDay': 0, 'strikePrice': 0, 'productId': {'symbol': 'HSAI', 'typeCode': 'EQUITY'}}</t>
+        </is>
+      </c>
+      <c r="Z36" t="inlineStr">
+        <is>
+          <t>{'lastTrade': 28.0638, 'lastTradeTime': 1757527580, 'change': -0.7262, 'changePct': -2.5224, 'volume': 1998515, 'quoteStatus': 'REALTIME'}</t>
+        </is>
+      </c>
+      <c r="AA36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>455519818900</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>EQT</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>1749528000000</v>
+      </c>
+      <c r="D37" t="n">
+        <v>53.3552</v>
+      </c>
+      <c r="E37" t="n">
+        <v>0</v>
+      </c>
+      <c r="F37" t="n">
+        <v>0</v>
+      </c>
+      <c r="G37" t="n">
+        <v>200</v>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>TYPE2</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="J37" t="n">
+        <v>126</v>
+      </c>
+      <c r="K37" t="n">
+        <v>1.2537</v>
+      </c>
+      <c r="L37" t="n">
+        <v>10176</v>
+      </c>
+      <c r="M37" t="n">
+        <v>10671.04</v>
+      </c>
+      <c r="N37" t="n">
+        <v>-495.04</v>
+      </c>
+      <c r="O37" t="n">
+        <v>-4.639</v>
+      </c>
+      <c r="P37" t="n">
+        <v>3.528</v>
+      </c>
+      <c r="Q37" t="n">
+        <v>53.3552</v>
+      </c>
+      <c r="R37" t="n">
+        <v>0</v>
+      </c>
+      <c r="S37" t="n">
+        <v>0</v>
+      </c>
+      <c r="T37" t="n">
+        <v>0</v>
+      </c>
+      <c r="U37" t="n">
+        <v>0</v>
+      </c>
+      <c r="V37" t="n">
+        <v>50.25</v>
+      </c>
+      <c r="W37" t="inlineStr">
+        <is>
+          <t>https://api.etrade.com/v1/accounts/fOTHyxD-9tctDlNfYkhFzA/portfolio/455519818900.json</t>
+        </is>
+      </c>
+      <c r="X37" t="inlineStr">
+        <is>
+          <t>https://api.etrade.com/v1/market/quote/EQT.json</t>
+        </is>
+      </c>
+      <c r="Y37" t="inlineStr">
+        <is>
+          <t>{'symbol': 'EQT', 'securityType': 'EQ', 'expiryYear': 0, 'expiryMonth': 0, 'expiryDay': 0, 'strikePrice': 0, 'productId': {'symbol': 'EQT', 'typeCode': 'EQUITY'}}</t>
+        </is>
+      </c>
+      <c r="Z37" t="inlineStr">
+        <is>
+          <t>{'lastTrade': 50.88, 'lastTradeTime': 1757527580, 'change': 0.63, 'changePct': 1.2537, 'volume': 2884712, 'quoteStatus': 'REALTIME'}</t>
+        </is>
+      </c>
+      <c r="AA37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>384696870900</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>EIC</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>1718164800000</v>
+      </c>
+      <c r="D38" t="n">
+        <v>15.65</v>
+      </c>
+      <c r="E38" t="n">
+        <v>0</v>
+      </c>
+      <c r="F38" t="n">
+        <v>0</v>
+      </c>
+      <c r="G38" t="n">
+        <v>466</v>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>TYPE2</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="J38" t="n">
+        <v>-15.9372</v>
+      </c>
+      <c r="K38" t="n">
+        <v>-0.26</v>
+      </c>
+      <c r="L38" t="n">
+        <v>6111.9628</v>
+      </c>
+      <c r="M38" t="n">
+        <v>7292.8999</v>
+      </c>
+      <c r="N38" t="n">
+        <v>-1180.9372</v>
+      </c>
+      <c r="O38" t="n">
+        <v>-16.1929</v>
+      </c>
+      <c r="P38" t="n">
+        <v>2.119</v>
+      </c>
+      <c r="Q38" t="n">
+        <v>15.65</v>
+      </c>
+      <c r="R38" t="n">
+        <v>0</v>
+      </c>
+      <c r="S38" t="n">
+        <v>0</v>
+      </c>
+      <c r="T38" t="n">
+        <v>0</v>
+      </c>
+      <c r="U38" t="n">
+        <v>0</v>
+      </c>
+      <c r="V38" t="n">
+        <v>13.15</v>
+      </c>
+      <c r="W38" t="inlineStr">
+        <is>
+          <t>https://api.etrade.com/v1/accounts/fOTHyxD-9tctDlNfYkhFzA/portfolio/384696870900.json</t>
+        </is>
+      </c>
+      <c r="X38" t="inlineStr">
+        <is>
+          <t>https://api.etrade.com/v1/market/quote/EIC.json</t>
+        </is>
+      </c>
+      <c r="Y38" t="inlineStr">
+        <is>
+          <t>{'symbol': 'EIC', 'securityType': 'EQ', 'securitySubType': 'CMUT', 'expiryYear': 0, 'expiryMonth': 0, 'expiryDay': 0, 'strikePrice': 0, 'productId': {'symbol': 'EIC', 'typeCode': 'EQUITY'}}</t>
+        </is>
+      </c>
+      <c r="Z38" t="inlineStr">
+        <is>
+          <t>{'lastTrade': 13.1158, 'lastTradeTime': 1757527546, 'change': -0.0342, 'changePct': -0.26, 'volume': 150869, 'quoteStatus': 'REALTIME'}</t>
+        </is>
+      </c>
+      <c r="AA38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>384160526900</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>ECC</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>1717992000000</v>
+      </c>
+      <c r="D39" t="n">
+        <v>9.813800000000001</v>
+      </c>
+      <c r="E39" t="n">
+        <v>0</v>
+      </c>
+      <c r="F39" t="n">
+        <v>0</v>
+      </c>
+      <c r="G39" t="n">
+        <v>1142</v>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>TYPE2</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>LONG</t>
+        </is>
+      </c>
+      <c r="J39" t="n">
+        <v>148.46</v>
+      </c>
+      <c r="K39" t="n">
+        <v>1.8571</v>
+      </c>
+      <c r="L39" t="n">
+        <v>8142.46</v>
+      </c>
+      <c r="M39" t="n">
+        <v>11207.3698</v>
+      </c>
+      <c r="N39" t="n">
+        <v>-3064.9098</v>
+      </c>
+      <c r="O39" t="n">
+        <v>-27.3472</v>
+      </c>
+      <c r="P39" t="n">
+        <v>2.823</v>
+      </c>
+      <c r="Q39" t="n">
+        <v>9.813800000000001</v>
+      </c>
+      <c r="R39" t="n">
+        <v>0</v>
+      </c>
+      <c r="S39" t="n">
+        <v>0</v>
+      </c>
+      <c r="T39" t="n">
+        <v>0</v>
+      </c>
+      <c r="U39" t="n">
+        <v>0</v>
+      </c>
+      <c r="V39" t="n">
+        <v>7</v>
+      </c>
+      <c r="W39" t="inlineStr">
+        <is>
+          <t>https://api.etrade.com/v1/accounts/fOTHyxD-9tctDlNfYkhFzA/portfolio/384160526900.json</t>
+        </is>
+      </c>
+      <c r="X39" t="inlineStr">
+        <is>
+          <t>https://api.etrade.com/v1/market/quote/ECC.json</t>
+        </is>
+      </c>
+      <c r="Y39" t="inlineStr">
+        <is>
+          <t>{'symbol': 'ECC', 'securityType': 'EQ', 'securitySubType': 'CMUT', 'expiryYear': 0, 'expiryMonth': 0, 'expiryDay': 0, 'strikePrice': 0, 'productId': {'symbol': 'ECC', 'typeCode': 'EQUITY'}}</t>
+        </is>
+      </c>
+      <c r="Z39" t="inlineStr">
+        <is>
+          <t>{'lastTrade': 7.13, 'lastTradeTime': 1757527585, 'change': 0.13, 'changePct': 1.8571, 'volume': 1421645, 'quoteStatus': 'REALTIME'}</t>
+        </is>
+      </c>
+      <c r="AA39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>8404759844</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>UGL Sep 19 '25 $39 Call</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>1756785600000</v>
+      </c>
+      <c r="D40" t="n">
+        <v>1</v>
+      </c>
+      <c r="E40" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F40" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="G40" t="n">
+        <v>-1</v>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>TYPE2</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>SHORT</t>
+        </is>
+      </c>
+      <c r="J40" t="n">
+        <v>-30</v>
+      </c>
+      <c r="K40" t="n">
+        <v>-12.9032</v>
+      </c>
+      <c r="L40" t="n">
+        <v>-262.5</v>
+      </c>
+      <c r="M40" t="n">
+        <v>-99.48</v>
+      </c>
+      <c r="N40" t="n">
+        <v>-163.02</v>
+      </c>
+      <c r="O40" t="n">
+        <v>-163.8721</v>
+      </c>
+      <c r="P40" t="n">
+        <v>-0.091</v>
+      </c>
+      <c r="Q40" t="n">
+        <v>0.9948</v>
+      </c>
+      <c r="R40" t="n">
+        <v>0</v>
+      </c>
+      <c r="S40" t="n">
+        <v>0</v>
+      </c>
+      <c r="T40" t="n">
+        <v>0</v>
+      </c>
+      <c r="U40" t="n">
+        <v>0</v>
+      </c>
+      <c r="V40" t="n">
+        <v>2.325</v>
+      </c>
+      <c r="W40" t="inlineStr">
+        <is>
+          <t>https://api.etrade.com/v1/accounts/fOTHyxD-9tctDlNfYkhFzA/portfolio/8404759844.json</t>
+        </is>
+      </c>
+      <c r="X40" t="inlineStr">
+        <is>
+          <t>https://api.etrade.com/v1/market/quote/UGL:2025:9:19:CALL:39.json</t>
+        </is>
+      </c>
+      <c r="Y40" t="inlineStr">
+        <is>
+          <t>{'symbol': 'UGL', 'securityType': 'OPTN', 'callPut': 'CALL', 'expiryYear': 2025, 'expiryMonth': 9, 'expiryDay': 19, 'strikePrice': 39, 'productId': {'symbol': 'UGL', 'typeCode': 'EQUITY'}}</t>
+        </is>
+      </c>
+      <c r="Z40" t="inlineStr">
+        <is>
+          <t>{'lastTrade': 2.62, 'lastTradeTime': 1757527573, 'change': 0.3, 'changePct': 12.9032, 'volume': 18, 'quoteStatus': 'REALTIME'}</t>
+        </is>
+      </c>
+      <c r="AA40" t="inlineStr">
+        <is>
+          <t>UGL---250919C00039000</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>